<commit_message>
Atualização de base — 08/06/2026 10:31
</commit_message>
<xml_diff>
--- a/dados/metas.xlsx
+++ b/dados/metas.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pedro.sa\Documents\dashboard-oportunidades\dados\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CA9C60BC-231E-40F1-8914-CBA45405E77C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3E1BDF74-1019-44C6-ADA7-F0D708365B92}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Plan1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Plan1!$A$1:$R$240</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Plan1!$A$1:$R$236</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="974" uniqueCount="80">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="958" uniqueCount="79">
   <si>
     <t>CÓD</t>
   </si>
@@ -207,9 +207,6 @@
   </si>
   <si>
     <t>MASTER GRAOS</t>
-  </si>
-  <si>
-    <t>MECANIZAÇÃO DO CAFÉ</t>
   </si>
   <si>
     <t>CARLOS.NUNES</t>
@@ -646,7 +643,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:R240"/>
+  <dimension ref="A1:R236"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.140625" style="4"/>
@@ -9228,7 +9225,7 @@
         <v>240035</v>
       </c>
       <c r="B154" s="4" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C154" s="4" t="s">
         <v>19</v>
@@ -9273,7 +9270,7 @@
         <v>6000002</v>
       </c>
       <c r="Q154" s="4" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="R154" s="4" t="s">
         <v>21</v>
@@ -9284,7 +9281,7 @@
         <v>240035</v>
       </c>
       <c r="B155" s="4" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C155" s="4" t="s">
         <v>23</v>
@@ -9329,7 +9326,7 @@
         <v>6</v>
       </c>
       <c r="Q155" s="4" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="R155" s="4" t="s">
         <v>21</v>
@@ -9340,7 +9337,7 @@
         <v>240035</v>
       </c>
       <c r="B156" s="4" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C156" s="4" t="s">
         <v>24</v>
@@ -9385,7 +9382,7 @@
         <v>6</v>
       </c>
       <c r="Q156" s="4" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="R156" s="4" t="s">
         <v>21</v>
@@ -9396,7 +9393,7 @@
         <v>240035</v>
       </c>
       <c r="B157" s="4" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C157" s="4" t="s">
         <v>28</v>
@@ -9441,7 +9438,7 @@
         <v>60</v>
       </c>
       <c r="Q157" s="4" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="R157" s="4" t="s">
         <v>21</v>
@@ -9452,7 +9449,7 @@
         <v>2417</v>
       </c>
       <c r="B158" s="4" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C158" s="4" t="s">
         <v>19</v>
@@ -9497,7 +9494,7 @@
         <v>4500000</v>
       </c>
       <c r="Q158" s="4" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="R158" s="4" t="s">
         <v>21</v>
@@ -9508,7 +9505,7 @@
         <v>2417</v>
       </c>
       <c r="B159" s="4" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C159" s="4" t="s">
         <v>23</v>
@@ -9553,7 +9550,7 @@
         <v>6</v>
       </c>
       <c r="Q159" s="4" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="R159" s="4" t="s">
         <v>21</v>
@@ -9564,7 +9561,7 @@
         <v>2417</v>
       </c>
       <c r="B160" s="4" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C160" s="4" t="s">
         <v>24</v>
@@ -9609,7 +9606,7 @@
         <v>6</v>
       </c>
       <c r="Q160" s="4" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="R160" s="4" t="s">
         <v>21</v>
@@ -9620,7 +9617,7 @@
         <v>2417</v>
       </c>
       <c r="B161" s="4" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C161" s="4" t="s">
         <v>28</v>
@@ -9665,7 +9662,7 @@
         <v>50</v>
       </c>
       <c r="Q161" s="4" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="R161" s="4" t="s">
         <v>21</v>
@@ -9676,7 +9673,7 @@
         <v>2425</v>
       </c>
       <c r="B162" s="4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C162" s="4" t="s">
         <v>19</v>
@@ -9721,7 +9718,7 @@
         <v>4500000</v>
       </c>
       <c r="Q162" s="4" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="R162" s="4" t="s">
         <v>21</v>
@@ -9732,7 +9729,7 @@
         <v>2425</v>
       </c>
       <c r="B163" s="4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C163" s="4" t="s">
         <v>23</v>
@@ -9777,7 +9774,7 @@
         <v>6</v>
       </c>
       <c r="Q163" s="4" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="R163" s="4" t="s">
         <v>21</v>
@@ -9788,7 +9785,7 @@
         <v>2425</v>
       </c>
       <c r="B164" s="4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C164" s="4" t="s">
         <v>24</v>
@@ -9833,7 +9830,7 @@
         <v>6</v>
       </c>
       <c r="Q164" s="4" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="R164" s="4" t="s">
         <v>21</v>
@@ -9844,7 +9841,7 @@
         <v>2425</v>
       </c>
       <c r="B165" s="4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C165" s="4" t="s">
         <v>28</v>
@@ -9889,7 +9886,7 @@
         <v>40</v>
       </c>
       <c r="Q165" s="4" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="R165" s="4" t="s">
         <v>21</v>
@@ -9900,7 +9897,7 @@
         <v>240048</v>
       </c>
       <c r="B166" s="4" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C166" s="4" t="s">
         <v>19</v>
@@ -9945,7 +9942,7 @@
         <v>2500000</v>
       </c>
       <c r="Q166" s="4" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="R166" s="4" t="s">
         <v>21</v>
@@ -9956,7 +9953,7 @@
         <v>240048</v>
       </c>
       <c r="B167" s="4" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C167" s="4" t="s">
         <v>23</v>
@@ -10001,7 +9998,7 @@
         <v>6</v>
       </c>
       <c r="Q167" s="4" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="R167" s="4" t="s">
         <v>21</v>
@@ -10012,7 +10009,7 @@
         <v>240048</v>
       </c>
       <c r="B168" s="4" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C168" s="4" t="s">
         <v>24</v>
@@ -10057,7 +10054,7 @@
         <v>6</v>
       </c>
       <c r="Q168" s="4" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="R168" s="4" t="s">
         <v>21</v>
@@ -10068,7 +10065,7 @@
         <v>240048</v>
       </c>
       <c r="B169" s="4" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C169" s="4" t="s">
         <v>28</v>
@@ -10113,7 +10110,7 @@
         <v>15</v>
       </c>
       <c r="Q169" s="4" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="R169" s="4" t="s">
         <v>21</v>
@@ -10124,7 +10121,7 @@
         <v>240060</v>
       </c>
       <c r="B170" s="4" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C170" s="4" t="s">
         <v>19</v>
@@ -10169,7 +10166,7 @@
         <v>1200002</v>
       </c>
       <c r="Q170" s="4" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="R170" s="4" t="s">
         <v>34</v>
@@ -10180,7 +10177,7 @@
         <v>240060</v>
       </c>
       <c r="B171" s="4" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C171" s="4" t="s">
         <v>23</v>
@@ -10225,7 +10222,7 @@
         <v>6</v>
       </c>
       <c r="Q171" s="4" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="R171" s="4" t="s">
         <v>34</v>
@@ -10236,7 +10233,7 @@
         <v>240060</v>
       </c>
       <c r="B172" s="4" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C172" s="4" t="s">
         <v>24</v>
@@ -10281,7 +10278,7 @@
         <v>6</v>
       </c>
       <c r="Q172" s="4" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="R172" s="4" t="s">
         <v>34</v>
@@ -10292,7 +10289,7 @@
         <v>240060</v>
       </c>
       <c r="B173" s="4" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C173" s="4" t="s">
         <v>28</v>
@@ -10337,7 +10334,7 @@
         <v>15</v>
       </c>
       <c r="Q173" s="4" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="R173" s="4" t="s">
         <v>34</v>
@@ -10348,7 +10345,7 @@
         <v>2419</v>
       </c>
       <c r="B174" s="4" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C174" s="4" t="s">
         <v>19</v>
@@ -10393,7 +10390,7 @@
         <v>3500001</v>
       </c>
       <c r="Q174" s="4" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="R174" s="4" t="s">
         <v>21</v>
@@ -10404,7 +10401,7 @@
         <v>2419</v>
       </c>
       <c r="B175" s="4" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C175" s="4" t="s">
         <v>23</v>
@@ -10449,7 +10446,7 @@
         <v>6</v>
       </c>
       <c r="Q175" s="4" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="R175" s="4" t="s">
         <v>21</v>
@@ -10460,7 +10457,7 @@
         <v>2419</v>
       </c>
       <c r="B176" s="4" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C176" s="4" t="s">
         <v>24</v>
@@ -10505,7 +10502,7 @@
         <v>6</v>
       </c>
       <c r="Q176" s="4" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="R176" s="4" t="s">
         <v>21</v>
@@ -10516,7 +10513,7 @@
         <v>2419</v>
       </c>
       <c r="B177" s="4" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C177" s="4" t="s">
         <v>28</v>
@@ -10561,7 +10558,7 @@
         <v>40</v>
       </c>
       <c r="Q177" s="4" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="R177" s="4" t="s">
         <v>21</v>
@@ -10572,7 +10569,7 @@
         <v>240058</v>
       </c>
       <c r="B178" s="4" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C178" s="4" t="s">
         <v>19</v>
@@ -10617,7 +10614,7 @@
         <v>2399999</v>
       </c>
       <c r="Q178" s="4" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="R178" s="4" t="s">
         <v>21</v>
@@ -10628,7 +10625,7 @@
         <v>240058</v>
       </c>
       <c r="B179" s="4" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C179" s="4" t="s">
         <v>23</v>
@@ -10673,7 +10670,7 @@
         <v>6</v>
       </c>
       <c r="Q179" s="4" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="R179" s="4" t="s">
         <v>21</v>
@@ -10684,7 +10681,7 @@
         <v>240058</v>
       </c>
       <c r="B180" s="4" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C180" s="4" t="s">
         <v>24</v>
@@ -10729,7 +10726,7 @@
         <v>6</v>
       </c>
       <c r="Q180" s="4" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="R180" s="4" t="s">
         <v>21</v>
@@ -10740,7 +10737,7 @@
         <v>240058</v>
       </c>
       <c r="B181" s="4" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C181" s="4" t="s">
         <v>28</v>
@@ -10785,7 +10782,7 @@
         <v>30</v>
       </c>
       <c r="Q181" s="4" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="R181" s="4" t="s">
         <v>21</v>
@@ -10796,7 +10793,7 @@
         <v>230305</v>
       </c>
       <c r="B182" s="4" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C182" s="4" t="s">
         <v>19</v>
@@ -10841,7 +10838,7 @@
         <v>4499999</v>
       </c>
       <c r="Q182" s="4" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="R182" s="4" t="s">
         <v>21</v>
@@ -10852,7 +10849,7 @@
         <v>230305</v>
       </c>
       <c r="B183" s="4" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C183" s="4" t="s">
         <v>23</v>
@@ -10897,7 +10894,7 @@
         <v>12</v>
       </c>
       <c r="Q183" s="4" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="R183" s="4" t="s">
         <v>21</v>
@@ -10908,7 +10905,7 @@
         <v>230305</v>
       </c>
       <c r="B184" s="4" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C184" s="4" t="s">
         <v>24</v>
@@ -10953,7 +10950,7 @@
         <v>5</v>
       </c>
       <c r="Q184" s="4" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="R184" s="4" t="s">
         <v>21</v>
@@ -10964,16 +10961,52 @@
         <v>230305</v>
       </c>
       <c r="B185" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="C185" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="D185" s="4">
+        <v>1</v>
+      </c>
+      <c r="E185" s="4">
+        <v>2</v>
+      </c>
+      <c r="F185" s="4">
+        <v>2</v>
+      </c>
+      <c r="G185" s="4">
+        <v>3</v>
+      </c>
+      <c r="H185" s="4">
+        <v>2</v>
+      </c>
+      <c r="I185" s="4">
+        <v>2</v>
+      </c>
+      <c r="J185" s="4">
+        <v>2</v>
+      </c>
+      <c r="K185" s="4">
+        <v>3</v>
+      </c>
+      <c r="L185" s="4">
+        <v>2</v>
+      </c>
+      <c r="M185" s="4">
+        <v>3</v>
+      </c>
+      <c r="N185" s="4">
+        <v>2</v>
+      </c>
+      <c r="O185" s="4">
+        <v>3</v>
+      </c>
+      <c r="P185" s="4">
+        <v>27</v>
+      </c>
+      <c r="Q185" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="C185" s="4" t="s">
-        <v>56</v>
-      </c>
-      <c r="P185" s="4">
-        <v>0</v>
-      </c>
-      <c r="Q185" s="4" t="s">
-        <v>66</v>
       </c>
       <c r="R185" s="4" t="s">
         <v>21</v>
@@ -10984,52 +11017,52 @@
         <v>230305</v>
       </c>
       <c r="B186" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="C186" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="D186" s="4">
+        <v>0</v>
+      </c>
+      <c r="E186" s="4">
+        <v>1</v>
+      </c>
+      <c r="F186" s="4">
+        <v>0</v>
+      </c>
+      <c r="G186" s="4">
+        <v>0</v>
+      </c>
+      <c r="H186" s="4">
+        <v>1</v>
+      </c>
+      <c r="I186" s="4">
+        <v>0</v>
+      </c>
+      <c r="J186" s="4">
+        <v>1</v>
+      </c>
+      <c r="K186" s="4">
+        <v>0</v>
+      </c>
+      <c r="L186" s="4">
+        <v>1</v>
+      </c>
+      <c r="M186" s="4">
+        <v>0</v>
+      </c>
+      <c r="N186" s="4">
+        <v>1</v>
+      </c>
+      <c r="O186" s="4">
+        <v>0</v>
+      </c>
+      <c r="P186" s="4">
+        <v>5</v>
+      </c>
+      <c r="Q186" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="C186" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="D186" s="4">
-        <v>1</v>
-      </c>
-      <c r="E186" s="4">
-        <v>2</v>
-      </c>
-      <c r="F186" s="4">
-        <v>2</v>
-      </c>
-      <c r="G186" s="4">
-        <v>3</v>
-      </c>
-      <c r="H186" s="4">
-        <v>2</v>
-      </c>
-      <c r="I186" s="4">
-        <v>2</v>
-      </c>
-      <c r="J186" s="4">
-        <v>2</v>
-      </c>
-      <c r="K186" s="4">
-        <v>3</v>
-      </c>
-      <c r="L186" s="4">
-        <v>2</v>
-      </c>
-      <c r="M186" s="4">
-        <v>3</v>
-      </c>
-      <c r="N186" s="4">
-        <v>2</v>
-      </c>
-      <c r="O186" s="4">
-        <v>3</v>
-      </c>
-      <c r="P186" s="4">
-        <v>27</v>
-      </c>
-      <c r="Q186" s="4" t="s">
-        <v>66</v>
       </c>
       <c r="R186" s="4" t="s">
         <v>21</v>
@@ -11037,55 +11070,55 @@
     </row>
     <row r="187" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A187" s="4">
-        <v>230305</v>
+        <v>230307</v>
       </c>
       <c r="B187" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="C187" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="D187" s="4">
+        <v>299114</v>
+      </c>
+      <c r="E187" s="4">
+        <v>319055</v>
+      </c>
+      <c r="F187" s="4">
+        <v>445347</v>
+      </c>
+      <c r="G187" s="4">
+        <v>458641</v>
+      </c>
+      <c r="H187" s="4">
+        <v>405465</v>
+      </c>
+      <c r="I187" s="4">
+        <v>438700</v>
+      </c>
+      <c r="J187" s="4">
+        <v>392171</v>
+      </c>
+      <c r="K187" s="4">
+        <v>438700</v>
+      </c>
+      <c r="L187" s="4">
+        <v>398818</v>
+      </c>
+      <c r="M187" s="4">
+        <v>252585</v>
+      </c>
+      <c r="N187" s="4">
+        <v>212703</v>
+      </c>
+      <c r="O187" s="4">
+        <v>438700</v>
+      </c>
+      <c r="P187" s="4">
+        <v>4499999</v>
+      </c>
+      <c r="Q187" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="C187" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="D187" s="4">
-        <v>0</v>
-      </c>
-      <c r="E187" s="4">
-        <v>1</v>
-      </c>
-      <c r="F187" s="4">
-        <v>0</v>
-      </c>
-      <c r="G187" s="4">
-        <v>0</v>
-      </c>
-      <c r="H187" s="4">
-        <v>1</v>
-      </c>
-      <c r="I187" s="4">
-        <v>0</v>
-      </c>
-      <c r="J187" s="4">
-        <v>1</v>
-      </c>
-      <c r="K187" s="4">
-        <v>0</v>
-      </c>
-      <c r="L187" s="4">
-        <v>1</v>
-      </c>
-      <c r="M187" s="4">
-        <v>0</v>
-      </c>
-      <c r="N187" s="4">
-        <v>1</v>
-      </c>
-      <c r="O187" s="4">
-        <v>0</v>
-      </c>
-      <c r="P187" s="4">
-        <v>5</v>
-      </c>
-      <c r="Q187" s="4" t="s">
-        <v>66</v>
       </c>
       <c r="R187" s="4" t="s">
         <v>21</v>
@@ -11096,52 +11129,52 @@
         <v>230307</v>
       </c>
       <c r="B188" s="4" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C188" s="4" t="s">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="D188" s="4">
-        <v>299114</v>
+        <v>1</v>
       </c>
       <c r="E188" s="4">
-        <v>319055</v>
+        <v>1</v>
       </c>
       <c r="F188" s="4">
-        <v>445347</v>
+        <v>1</v>
       </c>
       <c r="G188" s="4">
-        <v>458641</v>
+        <v>1</v>
       </c>
       <c r="H188" s="4">
-        <v>405465</v>
+        <v>1</v>
       </c>
       <c r="I188" s="4">
-        <v>438700</v>
+        <v>1</v>
       </c>
       <c r="J188" s="4">
-        <v>392171</v>
+        <v>1</v>
       </c>
       <c r="K188" s="4">
-        <v>438700</v>
+        <v>1</v>
       </c>
       <c r="L188" s="4">
-        <v>398818</v>
+        <v>1</v>
       </c>
       <c r="M188" s="4">
-        <v>252585</v>
+        <v>1</v>
       </c>
       <c r="N188" s="4">
-        <v>212703</v>
+        <v>1</v>
       </c>
       <c r="O188" s="4">
-        <v>438700</v>
+        <v>1</v>
       </c>
       <c r="P188" s="4">
-        <v>4499999</v>
+        <v>12</v>
       </c>
       <c r="Q188" s="4" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="R188" s="4" t="s">
         <v>21</v>
@@ -11152,52 +11185,52 @@
         <v>230307</v>
       </c>
       <c r="B189" s="4" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C189" s="4" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D189" s="4">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E189" s="4">
         <v>1</v>
       </c>
       <c r="F189" s="4">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G189" s="4">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H189" s="4">
         <v>1</v>
       </c>
       <c r="I189" s="4">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J189" s="4">
         <v>1</v>
       </c>
       <c r="K189" s="4">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L189" s="4">
         <v>1</v>
       </c>
       <c r="M189" s="4">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N189" s="4">
         <v>1</v>
       </c>
       <c r="O189" s="4">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P189" s="4">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="Q189" s="4" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="R189" s="4" t="s">
         <v>21</v>
@@ -11208,52 +11241,52 @@
         <v>230307</v>
       </c>
       <c r="B190" s="4" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C190" s="4" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="D190" s="4">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E190" s="4">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F190" s="4">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G190" s="4">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H190" s="4">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I190" s="4">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J190" s="4">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K190" s="4">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="L190" s="4">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M190" s="4">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="N190" s="4">
         <v>1</v>
       </c>
       <c r="O190" s="4">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="P190" s="4">
-        <v>5</v>
+        <v>23</v>
       </c>
       <c r="Q190" s="4" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="R190" s="4" t="s">
         <v>21</v>
@@ -11264,16 +11297,52 @@
         <v>230307</v>
       </c>
       <c r="B191" s="4" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C191" s="4" t="s">
-        <v>56</v>
+        <v>39</v>
+      </c>
+      <c r="D191" s="4">
+        <v>0</v>
+      </c>
+      <c r="E191" s="4">
+        <v>1</v>
+      </c>
+      <c r="F191" s="4">
+        <v>0</v>
+      </c>
+      <c r="G191" s="4">
+        <v>0</v>
+      </c>
+      <c r="H191" s="4">
+        <v>1</v>
+      </c>
+      <c r="I191" s="4">
+        <v>0</v>
+      </c>
+      <c r="J191" s="4">
+        <v>1</v>
+      </c>
+      <c r="K191" s="4">
+        <v>0</v>
+      </c>
+      <c r="L191" s="4">
+        <v>1</v>
+      </c>
+      <c r="M191" s="4">
+        <v>0</v>
+      </c>
+      <c r="N191" s="4">
+        <v>1</v>
+      </c>
+      <c r="O191" s="4">
+        <v>0</v>
       </c>
       <c r="P191" s="4">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="Q191" s="4" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="R191" s="4" t="s">
         <v>21</v>
@@ -11281,55 +11350,55 @@
     </row>
     <row r="192" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A192" s="4">
-        <v>230307</v>
+        <v>230306</v>
       </c>
       <c r="B192" s="4" t="s">
         <v>67</v>
       </c>
       <c r="C192" s="4" t="s">
-        <v>28</v>
+        <v>19</v>
       </c>
       <c r="D192" s="4">
-        <v>1</v>
+        <v>299114</v>
       </c>
       <c r="E192" s="4">
-        <v>2</v>
+        <v>319055</v>
       </c>
       <c r="F192" s="4">
-        <v>2</v>
+        <v>445347</v>
       </c>
       <c r="G192" s="4">
-        <v>2</v>
+        <v>458641</v>
       </c>
       <c r="H192" s="4">
-        <v>2</v>
+        <v>405465</v>
       </c>
       <c r="I192" s="4">
-        <v>2</v>
+        <v>438700</v>
       </c>
       <c r="J192" s="4">
-        <v>2</v>
+        <v>392171</v>
       </c>
       <c r="K192" s="4">
-        <v>3</v>
+        <v>438700</v>
       </c>
       <c r="L192" s="4">
-        <v>2</v>
+        <v>398818</v>
       </c>
       <c r="M192" s="4">
-        <v>2</v>
+        <v>252585</v>
       </c>
       <c r="N192" s="4">
-        <v>1</v>
+        <v>212703</v>
       </c>
       <c r="O192" s="4">
-        <v>2</v>
+        <v>438700</v>
       </c>
       <c r="P192" s="4">
-        <v>23</v>
+        <v>4499999</v>
       </c>
       <c r="Q192" s="4" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="R192" s="4" t="s">
         <v>21</v>
@@ -11337,55 +11406,55 @@
     </row>
     <row r="193" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A193" s="4">
-        <v>230307</v>
+        <v>230306</v>
       </c>
       <c r="B193" s="4" t="s">
         <v>67</v>
       </c>
       <c r="C193" s="4" t="s">
-        <v>39</v>
+        <v>23</v>
       </c>
       <c r="D193" s="4">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E193" s="4">
         <v>1</v>
       </c>
       <c r="F193" s="4">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G193" s="4">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H193" s="4">
         <v>1</v>
       </c>
       <c r="I193" s="4">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J193" s="4">
         <v>1</v>
       </c>
       <c r="K193" s="4">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L193" s="4">
         <v>1</v>
       </c>
       <c r="M193" s="4">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N193" s="4">
         <v>1</v>
       </c>
       <c r="O193" s="4">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P193" s="4">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="Q193" s="4" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="R193" s="4" t="s">
         <v>21</v>
@@ -11396,52 +11465,52 @@
         <v>230306</v>
       </c>
       <c r="B194" s="4" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C194" s="4" t="s">
-        <v>19</v>
+        <v>24</v>
       </c>
       <c r="D194" s="4">
-        <v>299114</v>
+        <v>0</v>
       </c>
       <c r="E194" s="4">
-        <v>319055</v>
+        <v>1</v>
       </c>
       <c r="F194" s="4">
-        <v>445347</v>
+        <v>0</v>
       </c>
       <c r="G194" s="4">
-        <v>458641</v>
+        <v>0</v>
       </c>
       <c r="H194" s="4">
-        <v>405465</v>
+        <v>1</v>
       </c>
       <c r="I194" s="4">
-        <v>438700</v>
+        <v>0</v>
       </c>
       <c r="J194" s="4">
-        <v>392171</v>
+        <v>1</v>
       </c>
       <c r="K194" s="4">
-        <v>438700</v>
+        <v>0</v>
       </c>
       <c r="L194" s="4">
-        <v>398818</v>
+        <v>1</v>
       </c>
       <c r="M194" s="4">
-        <v>252585</v>
+        <v>0</v>
       </c>
       <c r="N194" s="4">
-        <v>212703</v>
+        <v>1</v>
       </c>
       <c r="O194" s="4">
-        <v>438700</v>
+        <v>0</v>
       </c>
       <c r="P194" s="4">
-        <v>4499999</v>
+        <v>5</v>
       </c>
       <c r="Q194" s="4" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="R194" s="4" t="s">
         <v>21</v>
@@ -11452,52 +11521,52 @@
         <v>230306</v>
       </c>
       <c r="B195" s="4" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C195" s="4" t="s">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="D195" s="4">
         <v>1</v>
       </c>
       <c r="E195" s="4">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F195" s="4">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G195" s="4">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H195" s="4">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I195" s="4">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J195" s="4">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K195" s="4">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="L195" s="4">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M195" s="4">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N195" s="4">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O195" s="4">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="P195" s="4">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="Q195" s="4" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="R195" s="4" t="s">
         <v>21</v>
@@ -11508,10 +11577,10 @@
         <v>230306</v>
       </c>
       <c r="B196" s="4" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C196" s="4" t="s">
-        <v>24</v>
+        <v>39</v>
       </c>
       <c r="D196" s="4">
         <v>0</v>
@@ -11553,7 +11622,7 @@
         <v>5</v>
       </c>
       <c r="Q196" s="4" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="R196" s="4" t="s">
         <v>21</v>
@@ -11561,19 +11630,55 @@
     </row>
     <row r="197" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A197" s="4">
-        <v>230306</v>
+        <v>230301</v>
       </c>
       <c r="B197" s="4" t="s">
         <v>68</v>
       </c>
       <c r="C197" s="4" t="s">
-        <v>56</v>
+        <v>19</v>
+      </c>
+      <c r="D197" s="4">
+        <v>299114</v>
+      </c>
+      <c r="E197" s="4">
+        <v>319055</v>
+      </c>
+      <c r="F197" s="4">
+        <v>445347</v>
+      </c>
+      <c r="G197" s="4">
+        <v>458641</v>
+      </c>
+      <c r="H197" s="4">
+        <v>405465</v>
+      </c>
+      <c r="I197" s="4">
+        <v>438700</v>
+      </c>
+      <c r="J197" s="4">
+        <v>392171</v>
+      </c>
+      <c r="K197" s="4">
+        <v>438700</v>
+      </c>
+      <c r="L197" s="4">
+        <v>398818</v>
+      </c>
+      <c r="M197" s="4">
+        <v>252585</v>
+      </c>
+      <c r="N197" s="4">
+        <v>212703</v>
+      </c>
+      <c r="O197" s="4">
+        <v>438700</v>
       </c>
       <c r="P197" s="4">
-        <v>0</v>
+        <v>4499999</v>
       </c>
       <c r="Q197" s="4" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="R197" s="4" t="s">
         <v>21</v>
@@ -11581,55 +11686,55 @@
     </row>
     <row r="198" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A198" s="4">
-        <v>230306</v>
+        <v>230301</v>
       </c>
       <c r="B198" s="4" t="s">
         <v>68</v>
       </c>
       <c r="C198" s="4" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="D198" s="4">
         <v>1</v>
       </c>
       <c r="E198" s="4">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F198" s="4">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G198" s="4">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="H198" s="4">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I198" s="4">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J198" s="4">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K198" s="4">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="L198" s="4">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M198" s="4">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N198" s="4">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O198" s="4">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="P198" s="4">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="Q198" s="4" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="R198" s="4" t="s">
         <v>21</v>
@@ -11637,13 +11742,13 @@
     </row>
     <row r="199" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A199" s="4">
-        <v>230306</v>
+        <v>230301</v>
       </c>
       <c r="B199" s="4" t="s">
         <v>68</v>
       </c>
       <c r="C199" s="4" t="s">
-        <v>39</v>
+        <v>24</v>
       </c>
       <c r="D199" s="4">
         <v>0</v>
@@ -11685,7 +11790,7 @@
         <v>5</v>
       </c>
       <c r="Q199" s="4" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="R199" s="4" t="s">
         <v>21</v>
@@ -11696,52 +11801,52 @@
         <v>230301</v>
       </c>
       <c r="B200" s="4" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C200" s="4" t="s">
-        <v>19</v>
+        <v>28</v>
       </c>
       <c r="D200" s="4">
-        <v>299114</v>
+        <v>1</v>
       </c>
       <c r="E200" s="4">
-        <v>319055</v>
+        <v>2</v>
       </c>
       <c r="F200" s="4">
-        <v>445347</v>
+        <v>2</v>
       </c>
       <c r="G200" s="4">
-        <v>458641</v>
+        <v>3</v>
       </c>
       <c r="H200" s="4">
-        <v>405465</v>
+        <v>2</v>
       </c>
       <c r="I200" s="4">
-        <v>438700</v>
+        <v>2</v>
       </c>
       <c r="J200" s="4">
-        <v>392171</v>
+        <v>2</v>
       </c>
       <c r="K200" s="4">
-        <v>438700</v>
+        <v>3</v>
       </c>
       <c r="L200" s="4">
-        <v>398818</v>
+        <v>2</v>
       </c>
       <c r="M200" s="4">
-        <v>252585</v>
+        <v>3</v>
       </c>
       <c r="N200" s="4">
-        <v>212703</v>
+        <v>2</v>
       </c>
       <c r="O200" s="4">
-        <v>438700</v>
+        <v>3</v>
       </c>
       <c r="P200" s="4">
-        <v>4499999</v>
+        <v>27</v>
       </c>
       <c r="Q200" s="4" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="R200" s="4" t="s">
         <v>21</v>
@@ -11752,52 +11857,52 @@
         <v>230301</v>
       </c>
       <c r="B201" s="4" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C201" s="4" t="s">
-        <v>23</v>
+        <v>39</v>
       </c>
       <c r="D201" s="4">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E201" s="4">
         <v>1</v>
       </c>
       <c r="F201" s="4">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G201" s="4">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H201" s="4">
         <v>1</v>
       </c>
       <c r="I201" s="4">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J201" s="4">
         <v>1</v>
       </c>
       <c r="K201" s="4">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L201" s="4">
         <v>1</v>
       </c>
       <c r="M201" s="4">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N201" s="4">
         <v>1</v>
       </c>
       <c r="O201" s="4">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P201" s="4">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="Q201" s="4" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="R201" s="4" t="s">
         <v>21</v>
@@ -11805,55 +11910,55 @@
     </row>
     <row r="202" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A202" s="4">
-        <v>230301</v>
+        <v>280037</v>
       </c>
       <c r="B202" s="4" t="s">
         <v>69</v>
       </c>
       <c r="C202" s="4" t="s">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="D202" s="4">
-        <v>0</v>
+        <v>80233</v>
       </c>
       <c r="E202" s="4">
-        <v>1</v>
+        <v>132558</v>
       </c>
       <c r="F202" s="4">
-        <v>0</v>
+        <v>125581</v>
       </c>
       <c r="G202" s="4">
-        <v>0</v>
+        <v>102907</v>
       </c>
       <c r="H202" s="4">
-        <v>1</v>
+        <v>66279</v>
       </c>
       <c r="I202" s="4">
-        <v>0</v>
+        <v>125581</v>
       </c>
       <c r="J202" s="4">
-        <v>1</v>
+        <v>120349</v>
       </c>
       <c r="K202" s="4">
-        <v>0</v>
+        <v>162209</v>
       </c>
       <c r="L202" s="4">
-        <v>1</v>
+        <v>134302</v>
       </c>
       <c r="M202" s="4">
-        <v>0</v>
+        <v>139535</v>
       </c>
       <c r="N202" s="4">
-        <v>1</v>
+        <v>76745</v>
       </c>
       <c r="O202" s="4">
-        <v>0</v>
+        <v>83721</v>
       </c>
       <c r="P202" s="4">
-        <v>5</v>
+        <v>1350000</v>
       </c>
       <c r="Q202" s="4" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="R202" s="4" t="s">
         <v>21</v>
@@ -11861,19 +11966,55 @@
     </row>
     <row r="203" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A203" s="4">
-        <v>230301</v>
+        <v>280037</v>
       </c>
       <c r="B203" s="4" t="s">
         <v>69</v>
       </c>
       <c r="C203" s="4" t="s">
-        <v>56</v>
+        <v>22</v>
+      </c>
+      <c r="D203" s="4">
+        <v>0</v>
+      </c>
+      <c r="E203" s="4">
+        <v>1</v>
+      </c>
+      <c r="F203" s="4">
+        <v>0</v>
+      </c>
+      <c r="G203" s="4">
+        <v>0</v>
+      </c>
+      <c r="H203" s="4">
+        <v>0</v>
+      </c>
+      <c r="I203" s="4">
+        <v>0</v>
+      </c>
+      <c r="J203" s="4">
+        <v>0</v>
+      </c>
+      <c r="K203" s="4">
+        <v>0</v>
+      </c>
+      <c r="L203" s="4">
+        <v>0</v>
+      </c>
+      <c r="M203" s="4">
+        <v>0</v>
+      </c>
+      <c r="N203" s="4">
+        <v>0</v>
+      </c>
+      <c r="O203" s="4">
+        <v>0</v>
       </c>
       <c r="P203" s="4">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q203" s="4" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="R203" s="4" t="s">
         <v>21</v>
@@ -11881,55 +12022,55 @@
     </row>
     <row r="204" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A204" s="4">
-        <v>230301</v>
+        <v>280037</v>
       </c>
       <c r="B204" s="4" t="s">
         <v>69</v>
       </c>
       <c r="C204" s="4" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="D204" s="4">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E204" s="4">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F204" s="4">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G204" s="4">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="H204" s="4">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I204" s="4">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J204" s="4">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K204" s="4">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="L204" s="4">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M204" s="4">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N204" s="4">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="O204" s="4">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="P204" s="4">
-        <v>27</v>
+        <v>8</v>
       </c>
       <c r="Q204" s="4" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="R204" s="4" t="s">
         <v>21</v>
@@ -11937,13 +12078,13 @@
     </row>
     <row r="205" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A205" s="4">
-        <v>230301</v>
+        <v>280037</v>
       </c>
       <c r="B205" s="4" t="s">
         <v>69</v>
       </c>
       <c r="C205" s="4" t="s">
-        <v>39</v>
+        <v>24</v>
       </c>
       <c r="D205" s="4">
         <v>0</v>
@@ -11958,13 +12099,13 @@
         <v>0</v>
       </c>
       <c r="H205" s="4">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I205" s="4">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J205" s="4">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K205" s="4">
         <v>0</v>
@@ -11976,16 +12117,16 @@
         <v>0</v>
       </c>
       <c r="N205" s="4">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O205" s="4">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P205" s="4">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="Q205" s="4" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="R205" s="4" t="s">
         <v>21</v>
@@ -11996,52 +12137,52 @@
         <v>280037</v>
       </c>
       <c r="B206" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="C206" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="D206" s="4">
+        <v>0</v>
+      </c>
+      <c r="E206" s="4">
+        <v>0</v>
+      </c>
+      <c r="F206" s="4">
+        <v>0</v>
+      </c>
+      <c r="G206" s="4">
+        <v>0</v>
+      </c>
+      <c r="H206" s="4">
+        <v>0</v>
+      </c>
+      <c r="I206" s="4">
+        <v>0</v>
+      </c>
+      <c r="J206" s="4">
+        <v>0</v>
+      </c>
+      <c r="K206" s="4">
+        <v>0</v>
+      </c>
+      <c r="L206" s="4">
+        <v>0</v>
+      </c>
+      <c r="M206" s="4">
+        <v>1</v>
+      </c>
+      <c r="N206" s="4">
+        <v>0</v>
+      </c>
+      <c r="O206" s="4">
+        <v>0</v>
+      </c>
+      <c r="P206" s="4">
+        <v>1</v>
+      </c>
+      <c r="Q206" s="4" t="s">
         <v>70</v>
-      </c>
-      <c r="C206" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="D206" s="4">
-        <v>80233</v>
-      </c>
-      <c r="E206" s="4">
-        <v>132558</v>
-      </c>
-      <c r="F206" s="4">
-        <v>125581</v>
-      </c>
-      <c r="G206" s="4">
-        <v>102907</v>
-      </c>
-      <c r="H206" s="4">
-        <v>66279</v>
-      </c>
-      <c r="I206" s="4">
-        <v>125581</v>
-      </c>
-      <c r="J206" s="4">
-        <v>120349</v>
-      </c>
-      <c r="K206" s="4">
-        <v>162209</v>
-      </c>
-      <c r="L206" s="4">
-        <v>134302</v>
-      </c>
-      <c r="M206" s="4">
-        <v>139535</v>
-      </c>
-      <c r="N206" s="4">
-        <v>76745</v>
-      </c>
-      <c r="O206" s="4">
-        <v>83721</v>
-      </c>
-      <c r="P206" s="4">
-        <v>1350000</v>
-      </c>
-      <c r="Q206" s="4" t="s">
-        <v>71</v>
       </c>
       <c r="R206" s="4" t="s">
         <v>21</v>
@@ -12052,52 +12193,52 @@
         <v>280037</v>
       </c>
       <c r="B207" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="C207" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="D207" s="4">
+        <v>0</v>
+      </c>
+      <c r="E207" s="4">
+        <v>1</v>
+      </c>
+      <c r="F207" s="4">
+        <v>1</v>
+      </c>
+      <c r="G207" s="4">
+        <v>0</v>
+      </c>
+      <c r="H207" s="4">
+        <v>0</v>
+      </c>
+      <c r="I207" s="4">
+        <v>0</v>
+      </c>
+      <c r="J207" s="4">
+        <v>0</v>
+      </c>
+      <c r="K207" s="4">
+        <v>0</v>
+      </c>
+      <c r="L207" s="4">
+        <v>0</v>
+      </c>
+      <c r="M207" s="4">
+        <v>0</v>
+      </c>
+      <c r="N207" s="4">
+        <v>0</v>
+      </c>
+      <c r="O207" s="4">
+        <v>0</v>
+      </c>
+      <c r="P207" s="4">
+        <v>2</v>
+      </c>
+      <c r="Q207" s="4" t="s">
         <v>70</v>
-      </c>
-      <c r="C207" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="D207" s="4">
-        <v>0</v>
-      </c>
-      <c r="E207" s="4">
-        <v>1</v>
-      </c>
-      <c r="F207" s="4">
-        <v>0</v>
-      </c>
-      <c r="G207" s="4">
-        <v>0</v>
-      </c>
-      <c r="H207" s="4">
-        <v>0</v>
-      </c>
-      <c r="I207" s="4">
-        <v>0</v>
-      </c>
-      <c r="J207" s="4">
-        <v>0</v>
-      </c>
-      <c r="K207" s="4">
-        <v>0</v>
-      </c>
-      <c r="L207" s="4">
-        <v>0</v>
-      </c>
-      <c r="M207" s="4">
-        <v>0</v>
-      </c>
-      <c r="N207" s="4">
-        <v>0</v>
-      </c>
-      <c r="O207" s="4">
-        <v>0</v>
-      </c>
-      <c r="P207" s="4">
-        <v>1</v>
-      </c>
-      <c r="Q207" s="4" t="s">
-        <v>71</v>
       </c>
       <c r="R207" s="4" t="s">
         <v>21</v>
@@ -12108,52 +12249,52 @@
         <v>280037</v>
       </c>
       <c r="B208" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="C208" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="D208" s="4">
+        <v>0</v>
+      </c>
+      <c r="E208" s="4">
+        <v>0</v>
+      </c>
+      <c r="F208" s="4">
+        <v>0</v>
+      </c>
+      <c r="G208" s="4">
+        <v>0</v>
+      </c>
+      <c r="H208" s="4">
+        <v>0</v>
+      </c>
+      <c r="I208" s="4">
+        <v>0</v>
+      </c>
+      <c r="J208" s="4">
+        <v>0</v>
+      </c>
+      <c r="K208" s="4">
+        <v>0</v>
+      </c>
+      <c r="L208" s="4">
+        <v>1</v>
+      </c>
+      <c r="M208" s="4">
+        <v>0</v>
+      </c>
+      <c r="N208" s="4">
+        <v>0</v>
+      </c>
+      <c r="O208" s="4">
+        <v>0</v>
+      </c>
+      <c r="P208" s="4">
+        <v>1</v>
+      </c>
+      <c r="Q208" s="4" t="s">
         <v>70</v>
-      </c>
-      <c r="C208" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="D208" s="4">
-        <v>0</v>
-      </c>
-      <c r="E208" s="4">
-        <v>1</v>
-      </c>
-      <c r="F208" s="4">
-        <v>1</v>
-      </c>
-      <c r="G208" s="4">
-        <v>0</v>
-      </c>
-      <c r="H208" s="4">
-        <v>1</v>
-      </c>
-      <c r="I208" s="4">
-        <v>1</v>
-      </c>
-      <c r="J208" s="4">
-        <v>1</v>
-      </c>
-      <c r="K208" s="4">
-        <v>1</v>
-      </c>
-      <c r="L208" s="4">
-        <v>1</v>
-      </c>
-      <c r="M208" s="4">
-        <v>1</v>
-      </c>
-      <c r="N208" s="4">
-        <v>0</v>
-      </c>
-      <c r="O208" s="4">
-        <v>0</v>
-      </c>
-      <c r="P208" s="4">
-        <v>8</v>
-      </c>
-      <c r="Q208" s="4" t="s">
-        <v>71</v>
       </c>
       <c r="R208" s="4" t="s">
         <v>21</v>
@@ -12164,52 +12305,52 @@
         <v>280037</v>
       </c>
       <c r="B209" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="C209" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="D209" s="4">
+        <v>1</v>
+      </c>
+      <c r="E209" s="4">
+        <v>1</v>
+      </c>
+      <c r="F209" s="4">
+        <v>1</v>
+      </c>
+      <c r="G209" s="4">
+        <v>1</v>
+      </c>
+      <c r="H209" s="4">
+        <v>1</v>
+      </c>
+      <c r="I209" s="4">
+        <v>1</v>
+      </c>
+      <c r="J209" s="4">
+        <v>1</v>
+      </c>
+      <c r="K209" s="4">
+        <v>1</v>
+      </c>
+      <c r="L209" s="4">
+        <v>1</v>
+      </c>
+      <c r="M209" s="4">
+        <v>1</v>
+      </c>
+      <c r="N209" s="4">
+        <v>1</v>
+      </c>
+      <c r="O209" s="4">
+        <v>1</v>
+      </c>
+      <c r="P209" s="4">
+        <v>12</v>
+      </c>
+      <c r="Q209" s="4" t="s">
         <v>70</v>
-      </c>
-      <c r="C209" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="D209" s="4">
-        <v>0</v>
-      </c>
-      <c r="E209" s="4">
-        <v>1</v>
-      </c>
-      <c r="F209" s="4">
-        <v>0</v>
-      </c>
-      <c r="G209" s="4">
-        <v>0</v>
-      </c>
-      <c r="H209" s="4">
-        <v>0</v>
-      </c>
-      <c r="I209" s="4">
-        <v>1</v>
-      </c>
-      <c r="J209" s="4">
-        <v>0</v>
-      </c>
-      <c r="K209" s="4">
-        <v>0</v>
-      </c>
-      <c r="L209" s="4">
-        <v>1</v>
-      </c>
-      <c r="M209" s="4">
-        <v>0</v>
-      </c>
-      <c r="N209" s="4">
-        <v>0</v>
-      </c>
-      <c r="O209" s="4">
-        <v>1</v>
-      </c>
-      <c r="P209" s="4">
-        <v>4</v>
-      </c>
-      <c r="Q209" s="4" t="s">
-        <v>71</v>
       </c>
       <c r="R209" s="4" t="s">
         <v>21</v>
@@ -12220,52 +12361,52 @@
         <v>280037</v>
       </c>
       <c r="B210" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="C210" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="D210" s="4">
+        <v>95090</v>
+      </c>
+      <c r="E210" s="4">
+        <v>157106</v>
+      </c>
+      <c r="F210" s="4">
+        <v>148837</v>
+      </c>
+      <c r="G210" s="4">
+        <v>121964</v>
+      </c>
+      <c r="H210" s="4">
+        <v>78553</v>
+      </c>
+      <c r="I210" s="4">
+        <v>148837</v>
+      </c>
+      <c r="J210" s="4">
+        <v>142636</v>
+      </c>
+      <c r="K210" s="4">
+        <v>192248</v>
+      </c>
+      <c r="L210" s="4">
+        <v>159173</v>
+      </c>
+      <c r="M210" s="4">
+        <v>165375</v>
+      </c>
+      <c r="N210" s="4">
+        <v>90956</v>
+      </c>
+      <c r="O210" s="4">
+        <v>99225</v>
+      </c>
+      <c r="P210" s="4">
+        <v>1600000</v>
+      </c>
+      <c r="Q210" s="4" t="s">
         <v>70</v>
-      </c>
-      <c r="C210" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="D210" s="4">
-        <v>0</v>
-      </c>
-      <c r="E210" s="4">
-        <v>0</v>
-      </c>
-      <c r="F210" s="4">
-        <v>0</v>
-      </c>
-      <c r="G210" s="4">
-        <v>0</v>
-      </c>
-      <c r="H210" s="4">
-        <v>0</v>
-      </c>
-      <c r="I210" s="4">
-        <v>0</v>
-      </c>
-      <c r="J210" s="4">
-        <v>0</v>
-      </c>
-      <c r="K210" s="4">
-        <v>0</v>
-      </c>
-      <c r="L210" s="4">
-        <v>0</v>
-      </c>
-      <c r="M210" s="4">
-        <v>1</v>
-      </c>
-      <c r="N210" s="4">
-        <v>0</v>
-      </c>
-      <c r="O210" s="4">
-        <v>0</v>
-      </c>
-      <c r="P210" s="4">
-        <v>1</v>
-      </c>
-      <c r="Q210" s="4" t="s">
-        <v>71</v>
       </c>
       <c r="R210" s="4" t="s">
         <v>21</v>
@@ -12273,55 +12414,55 @@
     </row>
     <row r="211" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A211" s="4">
-        <v>280037</v>
+        <v>2712</v>
       </c>
       <c r="B211" s="4" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C211" s="4" t="s">
-        <v>26</v>
+        <v>19</v>
       </c>
       <c r="D211" s="4">
-        <v>0</v>
+        <v>100000</v>
       </c>
       <c r="E211" s="4">
-        <v>1</v>
+        <v>100000</v>
       </c>
       <c r="F211" s="4">
-        <v>1</v>
+        <v>200000</v>
       </c>
       <c r="G211" s="4">
-        <v>0</v>
+        <v>300000</v>
       </c>
       <c r="H211" s="4">
-        <v>0</v>
+        <v>100000</v>
       </c>
       <c r="I211" s="4">
-        <v>0</v>
+        <v>100000</v>
       </c>
       <c r="J211" s="4">
-        <v>0</v>
+        <v>200000</v>
       </c>
       <c r="K211" s="4">
-        <v>0</v>
+        <v>200000</v>
       </c>
       <c r="L211" s="4">
-        <v>0</v>
+        <v>300000</v>
       </c>
       <c r="M211" s="4">
-        <v>0</v>
+        <v>200000</v>
       </c>
       <c r="N211" s="4">
-        <v>0</v>
+        <v>200000</v>
       </c>
       <c r="O211" s="4">
-        <v>0</v>
+        <v>200000</v>
       </c>
       <c r="P211" s="4">
-        <v>2</v>
+        <v>2200000</v>
       </c>
       <c r="Q211" s="4" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="R211" s="4" t="s">
         <v>21</v>
@@ -12329,55 +12470,55 @@
     </row>
     <row r="212" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A212" s="4">
-        <v>280037</v>
+        <v>2712</v>
       </c>
       <c r="B212" s="4" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C212" s="4" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="D212" s="4">
         <v>0</v>
       </c>
       <c r="E212" s="4">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F212" s="4">
         <v>0</v>
       </c>
       <c r="G212" s="4">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H212" s="4">
         <v>0</v>
       </c>
       <c r="I212" s="4">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J212" s="4">
         <v>0</v>
       </c>
       <c r="K212" s="4">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L212" s="4">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M212" s="4">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N212" s="4">
         <v>0</v>
       </c>
       <c r="O212" s="4">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P212" s="4">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="Q212" s="4" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="R212" s="4" t="s">
         <v>21</v>
@@ -12385,55 +12526,55 @@
     </row>
     <row r="213" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A213" s="4">
-        <v>280037</v>
+        <v>2712</v>
       </c>
       <c r="B213" s="4" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C213" s="4" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="D213" s="4">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E213" s="4">
         <v>1</v>
       </c>
       <c r="F213" s="4">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G213" s="4">
         <v>1</v>
       </c>
       <c r="H213" s="4">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I213" s="4">
         <v>1</v>
       </c>
       <c r="J213" s="4">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K213" s="4">
         <v>1</v>
       </c>
       <c r="L213" s="4">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M213" s="4">
         <v>1</v>
       </c>
       <c r="N213" s="4">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O213" s="4">
         <v>1</v>
       </c>
       <c r="P213" s="4">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="Q213" s="4" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="R213" s="4" t="s">
         <v>21</v>
@@ -12441,55 +12582,55 @@
     </row>
     <row r="214" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A214" s="4">
-        <v>280037</v>
+        <v>2712</v>
       </c>
       <c r="B214" s="4" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C214" s="4" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D214" s="4">
-        <v>95090</v>
+        <v>1</v>
       </c>
       <c r="E214" s="4">
-        <v>157106</v>
+        <v>1</v>
       </c>
       <c r="F214" s="4">
-        <v>148837</v>
+        <v>2</v>
       </c>
       <c r="G214" s="4">
-        <v>121964</v>
+        <v>3</v>
       </c>
       <c r="H214" s="4">
-        <v>78553</v>
+        <v>1</v>
       </c>
       <c r="I214" s="4">
-        <v>148837</v>
+        <v>1</v>
       </c>
       <c r="J214" s="4">
-        <v>142636</v>
+        <v>1</v>
       </c>
       <c r="K214" s="4">
-        <v>192248</v>
+        <v>2</v>
       </c>
       <c r="L214" s="4">
-        <v>159173</v>
+        <v>3</v>
       </c>
       <c r="M214" s="4">
-        <v>165375</v>
+        <v>1</v>
       </c>
       <c r="N214" s="4">
-        <v>90956</v>
+        <v>2</v>
       </c>
       <c r="O214" s="4">
-        <v>99225</v>
+        <v>2</v>
       </c>
       <c r="P214" s="4">
-        <v>1600000</v>
+        <v>20</v>
       </c>
       <c r="Q214" s="4" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="R214" s="4" t="s">
         <v>21</v>
@@ -12500,52 +12641,52 @@
         <v>2712</v>
       </c>
       <c r="B215" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="C215" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="D215" s="4">
+        <v>0</v>
+      </c>
+      <c r="E215" s="4">
+        <v>0</v>
+      </c>
+      <c r="F215" s="4">
+        <v>1</v>
+      </c>
+      <c r="G215" s="4">
+        <v>0</v>
+      </c>
+      <c r="H215" s="4">
+        <v>0</v>
+      </c>
+      <c r="I215" s="4">
+        <v>1</v>
+      </c>
+      <c r="J215" s="4">
+        <v>0</v>
+      </c>
+      <c r="K215" s="4">
+        <v>0</v>
+      </c>
+      <c r="L215" s="4">
+        <v>1</v>
+      </c>
+      <c r="M215" s="4">
+        <v>0</v>
+      </c>
+      <c r="N215" s="4">
+        <v>0</v>
+      </c>
+      <c r="O215" s="4">
+        <v>1</v>
+      </c>
+      <c r="P215" s="4">
+        <v>4</v>
+      </c>
+      <c r="Q215" s="4" t="s">
         <v>72</v>
-      </c>
-      <c r="C215" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="D215" s="4">
-        <v>100000</v>
-      </c>
-      <c r="E215" s="4">
-        <v>100000</v>
-      </c>
-      <c r="F215" s="4">
-        <v>200000</v>
-      </c>
-      <c r="G215" s="4">
-        <v>300000</v>
-      </c>
-      <c r="H215" s="4">
-        <v>100000</v>
-      </c>
-      <c r="I215" s="4">
-        <v>100000</v>
-      </c>
-      <c r="J215" s="4">
-        <v>200000</v>
-      </c>
-      <c r="K215" s="4">
-        <v>200000</v>
-      </c>
-      <c r="L215" s="4">
-        <v>300000</v>
-      </c>
-      <c r="M215" s="4">
-        <v>200000</v>
-      </c>
-      <c r="N215" s="4">
-        <v>200000</v>
-      </c>
-      <c r="O215" s="4">
-        <v>200000</v>
-      </c>
-      <c r="P215" s="4">
-        <v>2200000</v>
-      </c>
-      <c r="Q215" s="4" t="s">
-        <v>73</v>
       </c>
       <c r="R215" s="4" t="s">
         <v>21</v>
@@ -12553,55 +12694,55 @@
     </row>
     <row r="216" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A216" s="4">
-        <v>2712</v>
+        <v>270018</v>
       </c>
       <c r="B216" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="C216" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="D216" s="4">
+        <v>0</v>
+      </c>
+      <c r="E216" s="4">
+        <v>0</v>
+      </c>
+      <c r="F216" s="4">
+        <v>200000</v>
+      </c>
+      <c r="G216" s="4">
+        <v>100000</v>
+      </c>
+      <c r="H216" s="4">
+        <v>100000</v>
+      </c>
+      <c r="I216" s="4">
+        <v>100000</v>
+      </c>
+      <c r="J216" s="4">
+        <v>200000</v>
+      </c>
+      <c r="K216" s="4">
+        <v>200000</v>
+      </c>
+      <c r="L216" s="4">
+        <v>200000</v>
+      </c>
+      <c r="M216" s="4">
+        <v>200000</v>
+      </c>
+      <c r="N216" s="4">
+        <v>100000</v>
+      </c>
+      <c r="O216" s="4">
+        <v>100000</v>
+      </c>
+      <c r="P216" s="4">
+        <v>1500000</v>
+      </c>
+      <c r="Q216" s="4" t="s">
         <v>72</v>
-      </c>
-      <c r="C216" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="D216" s="4">
-        <v>0</v>
-      </c>
-      <c r="E216" s="4">
-        <v>1</v>
-      </c>
-      <c r="F216" s="4">
-        <v>0</v>
-      </c>
-      <c r="G216" s="4">
-        <v>1</v>
-      </c>
-      <c r="H216" s="4">
-        <v>0</v>
-      </c>
-      <c r="I216" s="4">
-        <v>1</v>
-      </c>
-      <c r="J216" s="4">
-        <v>0</v>
-      </c>
-      <c r="K216" s="4">
-        <v>1</v>
-      </c>
-      <c r="L216" s="4">
-        <v>0</v>
-      </c>
-      <c r="M216" s="4">
-        <v>1</v>
-      </c>
-      <c r="N216" s="4">
-        <v>0</v>
-      </c>
-      <c r="O216" s="4">
-        <v>1</v>
-      </c>
-      <c r="P216" s="4">
-        <v>6</v>
-      </c>
-      <c r="Q216" s="4" t="s">
-        <v>73</v>
       </c>
       <c r="R216" s="4" t="s">
         <v>21</v>
@@ -12609,55 +12750,55 @@
     </row>
     <row r="217" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A217" s="4">
-        <v>2712</v>
+        <v>270018</v>
       </c>
       <c r="B217" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="C217" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="D217" s="4">
+        <v>0</v>
+      </c>
+      <c r="E217" s="4">
+        <v>0</v>
+      </c>
+      <c r="F217" s="4">
+        <v>0</v>
+      </c>
+      <c r="G217" s="4">
+        <v>1</v>
+      </c>
+      <c r="H217" s="4">
+        <v>0</v>
+      </c>
+      <c r="I217" s="4">
+        <v>1</v>
+      </c>
+      <c r="J217" s="4">
+        <v>0</v>
+      </c>
+      <c r="K217" s="4">
+        <v>1</v>
+      </c>
+      <c r="L217" s="4">
+        <v>0</v>
+      </c>
+      <c r="M217" s="4">
+        <v>1</v>
+      </c>
+      <c r="N217" s="4">
+        <v>0</v>
+      </c>
+      <c r="O217" s="4">
+        <v>1</v>
+      </c>
+      <c r="P217" s="4">
+        <v>5</v>
+      </c>
+      <c r="Q217" s="4" t="s">
         <v>72</v>
-      </c>
-      <c r="C217" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="D217" s="4">
-        <v>0</v>
-      </c>
-      <c r="E217" s="4">
-        <v>1</v>
-      </c>
-      <c r="F217" s="4">
-        <v>0</v>
-      </c>
-      <c r="G217" s="4">
-        <v>1</v>
-      </c>
-      <c r="H217" s="4">
-        <v>0</v>
-      </c>
-      <c r="I217" s="4">
-        <v>1</v>
-      </c>
-      <c r="J217" s="4">
-        <v>0</v>
-      </c>
-      <c r="K217" s="4">
-        <v>1</v>
-      </c>
-      <c r="L217" s="4">
-        <v>0</v>
-      </c>
-      <c r="M217" s="4">
-        <v>1</v>
-      </c>
-      <c r="N217" s="4">
-        <v>0</v>
-      </c>
-      <c r="O217" s="4">
-        <v>1</v>
-      </c>
-      <c r="P217" s="4">
-        <v>6</v>
-      </c>
-      <c r="Q217" s="4" t="s">
-        <v>73</v>
       </c>
       <c r="R217" s="4" t="s">
         <v>21</v>
@@ -12665,55 +12806,55 @@
     </row>
     <row r="218" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A218" s="4">
-        <v>2712</v>
+        <v>270018</v>
       </c>
       <c r="B218" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="C218" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="D218" s="4">
+        <v>0</v>
+      </c>
+      <c r="E218" s="4">
+        <v>0</v>
+      </c>
+      <c r="F218" s="4">
+        <v>0</v>
+      </c>
+      <c r="G218" s="4">
+        <v>1</v>
+      </c>
+      <c r="H218" s="4">
+        <v>0</v>
+      </c>
+      <c r="I218" s="4">
+        <v>1</v>
+      </c>
+      <c r="J218" s="4">
+        <v>0</v>
+      </c>
+      <c r="K218" s="4">
+        <v>0</v>
+      </c>
+      <c r="L218" s="4">
+        <v>0</v>
+      </c>
+      <c r="M218" s="4">
+        <v>1</v>
+      </c>
+      <c r="N218" s="4">
+        <v>0</v>
+      </c>
+      <c r="O218" s="4">
+        <v>1</v>
+      </c>
+      <c r="P218" s="4">
+        <v>4</v>
+      </c>
+      <c r="Q218" s="4" t="s">
         <v>72</v>
-      </c>
-      <c r="C218" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="D218" s="4">
-        <v>1</v>
-      </c>
-      <c r="E218" s="4">
-        <v>1</v>
-      </c>
-      <c r="F218" s="4">
-        <v>2</v>
-      </c>
-      <c r="G218" s="4">
-        <v>3</v>
-      </c>
-      <c r="H218" s="4">
-        <v>1</v>
-      </c>
-      <c r="I218" s="4">
-        <v>1</v>
-      </c>
-      <c r="J218" s="4">
-        <v>1</v>
-      </c>
-      <c r="K218" s="4">
-        <v>2</v>
-      </c>
-      <c r="L218" s="4">
-        <v>3</v>
-      </c>
-      <c r="M218" s="4">
-        <v>1</v>
-      </c>
-      <c r="N218" s="4">
-        <v>2</v>
-      </c>
-      <c r="O218" s="4">
-        <v>2</v>
-      </c>
-      <c r="P218" s="4">
-        <v>20</v>
-      </c>
-      <c r="Q218" s="4" t="s">
-        <v>73</v>
       </c>
       <c r="R218" s="4" t="s">
         <v>21</v>
@@ -12721,55 +12862,55 @@
     </row>
     <row r="219" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A219" s="4">
-        <v>2712</v>
+        <v>270018</v>
       </c>
       <c r="B219" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="C219" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="D219" s="4">
+        <v>0</v>
+      </c>
+      <c r="E219" s="4">
+        <v>0</v>
+      </c>
+      <c r="F219" s="4">
+        <v>1</v>
+      </c>
+      <c r="G219" s="4">
+        <v>1</v>
+      </c>
+      <c r="H219" s="4">
+        <v>1</v>
+      </c>
+      <c r="I219" s="4">
+        <v>1</v>
+      </c>
+      <c r="J219" s="4">
+        <v>1</v>
+      </c>
+      <c r="K219" s="4">
+        <v>1</v>
+      </c>
+      <c r="L219" s="4">
+        <v>1</v>
+      </c>
+      <c r="M219" s="4">
+        <v>1</v>
+      </c>
+      <c r="N219" s="4">
+        <v>1</v>
+      </c>
+      <c r="O219" s="4">
+        <v>1</v>
+      </c>
+      <c r="P219" s="4">
+        <v>10</v>
+      </c>
+      <c r="Q219" s="4" t="s">
         <v>72</v>
-      </c>
-      <c r="C219" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="D219" s="4">
-        <v>0</v>
-      </c>
-      <c r="E219" s="4">
-        <v>0</v>
-      </c>
-      <c r="F219" s="4">
-        <v>1</v>
-      </c>
-      <c r="G219" s="4">
-        <v>0</v>
-      </c>
-      <c r="H219" s="4">
-        <v>0</v>
-      </c>
-      <c r="I219" s="4">
-        <v>1</v>
-      </c>
-      <c r="J219" s="4">
-        <v>0</v>
-      </c>
-      <c r="K219" s="4">
-        <v>0</v>
-      </c>
-      <c r="L219" s="4">
-        <v>1</v>
-      </c>
-      <c r="M219" s="4">
-        <v>0</v>
-      </c>
-      <c r="N219" s="4">
-        <v>0</v>
-      </c>
-      <c r="O219" s="4">
-        <v>1</v>
-      </c>
-      <c r="P219" s="4">
-        <v>4</v>
-      </c>
-      <c r="Q219" s="4" t="s">
-        <v>73</v>
       </c>
       <c r="R219" s="4" t="s">
         <v>21</v>
@@ -12780,10 +12921,10 @@
         <v>270018</v>
       </c>
       <c r="B220" s="4" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C220" s="4" t="s">
-        <v>19</v>
+        <v>39</v>
       </c>
       <c r="D220" s="4">
         <v>0</v>
@@ -12792,40 +12933,40 @@
         <v>0</v>
       </c>
       <c r="F220" s="4">
-        <v>200000</v>
+        <v>1</v>
       </c>
       <c r="G220" s="4">
-        <v>100000</v>
+        <v>0</v>
       </c>
       <c r="H220" s="4">
-        <v>100000</v>
+        <v>0</v>
       </c>
       <c r="I220" s="4">
-        <v>100000</v>
+        <v>1</v>
       </c>
       <c r="J220" s="4">
-        <v>200000</v>
+        <v>0</v>
       </c>
       <c r="K220" s="4">
-        <v>200000</v>
+        <v>0</v>
       </c>
       <c r="L220" s="4">
-        <v>200000</v>
+        <v>1</v>
       </c>
       <c r="M220" s="4">
-        <v>200000</v>
+        <v>0</v>
       </c>
       <c r="N220" s="4">
-        <v>100000</v>
+        <v>0</v>
       </c>
       <c r="O220" s="4">
-        <v>100000</v>
+        <v>1</v>
       </c>
       <c r="P220" s="4">
-        <v>1500000</v>
+        <v>4</v>
       </c>
       <c r="Q220" s="4" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="R220" s="4" t="s">
         <v>21</v>
@@ -12833,55 +12974,55 @@
     </row>
     <row r="221" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A221" s="4">
-        <v>270018</v>
+        <v>270035</v>
       </c>
       <c r="B221" s="4" t="s">
         <v>74</v>
       </c>
       <c r="C221" s="4" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="D221" s="4">
-        <v>0</v>
+        <v>100000</v>
       </c>
       <c r="E221" s="4">
-        <v>0</v>
+        <v>100000</v>
       </c>
       <c r="F221" s="4">
-        <v>0</v>
+        <v>200000</v>
       </c>
       <c r="G221" s="4">
-        <v>1</v>
+        <v>100000</v>
       </c>
       <c r="H221" s="4">
-        <v>0</v>
+        <v>100000</v>
       </c>
       <c r="I221" s="4">
-        <v>1</v>
+        <v>100000</v>
       </c>
       <c r="J221" s="4">
-        <v>0</v>
+        <v>200000</v>
       </c>
       <c r="K221" s="4">
-        <v>1</v>
+        <v>200000</v>
       </c>
       <c r="L221" s="4">
-        <v>0</v>
+        <v>200000</v>
       </c>
       <c r="M221" s="4">
-        <v>1</v>
+        <v>200000</v>
       </c>
       <c r="N221" s="4">
-        <v>0</v>
+        <v>100000</v>
       </c>
       <c r="O221" s="4">
-        <v>1</v>
+        <v>100000</v>
       </c>
       <c r="P221" s="4">
-        <v>5</v>
+        <v>1700000</v>
       </c>
       <c r="Q221" s="4" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="R221" s="4" t="s">
         <v>21</v>
@@ -12889,19 +13030,19 @@
     </row>
     <row r="222" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A222" s="4">
-        <v>270018</v>
+        <v>270035</v>
       </c>
       <c r="B222" s="4" t="s">
         <v>74</v>
       </c>
       <c r="C222" s="4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D222" s="4">
         <v>0</v>
       </c>
       <c r="E222" s="4">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F222" s="4">
         <v>0</v>
@@ -12919,7 +13060,7 @@
         <v>0</v>
       </c>
       <c r="K222" s="4">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L222" s="4">
         <v>0</v>
@@ -12934,10 +13075,10 @@
         <v>1</v>
       </c>
       <c r="P222" s="4">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="Q222" s="4" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="R222" s="4" t="s">
         <v>21</v>
@@ -12945,55 +13086,55 @@
     </row>
     <row r="223" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A223" s="4">
-        <v>270018</v>
+        <v>270035</v>
       </c>
       <c r="B223" s="4" t="s">
         <v>74</v>
       </c>
       <c r="C223" s="4" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="D223" s="4">
         <v>0</v>
       </c>
       <c r="E223" s="4">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F223" s="4">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G223" s="4">
         <v>1</v>
       </c>
       <c r="H223" s="4">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I223" s="4">
         <v>1</v>
       </c>
       <c r="J223" s="4">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K223" s="4">
         <v>1</v>
       </c>
       <c r="L223" s="4">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M223" s="4">
         <v>1</v>
       </c>
       <c r="N223" s="4">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O223" s="4">
         <v>1</v>
       </c>
       <c r="P223" s="4">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="Q223" s="4" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="R223" s="4" t="s">
         <v>21</v>
@@ -13001,55 +13142,55 @@
     </row>
     <row r="224" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A224" s="4">
-        <v>270018</v>
+        <v>270035</v>
       </c>
       <c r="B224" s="4" t="s">
         <v>74</v>
       </c>
       <c r="C224" s="4" t="s">
-        <v>39</v>
+        <v>28</v>
       </c>
       <c r="D224" s="4">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E224" s="4">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F224" s="4">
         <v>1</v>
       </c>
       <c r="G224" s="4">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H224" s="4">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I224" s="4">
         <v>1</v>
       </c>
       <c r="J224" s="4">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K224" s="4">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L224" s="4">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M224" s="4">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N224" s="4">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O224" s="4">
         <v>1</v>
       </c>
       <c r="P224" s="4">
-        <v>4</v>
+        <v>13</v>
       </c>
       <c r="Q224" s="4" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="R224" s="4" t="s">
         <v>21</v>
@@ -13060,52 +13201,52 @@
         <v>270035</v>
       </c>
       <c r="B225" s="4" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C225" s="4" t="s">
-        <v>19</v>
+        <v>39</v>
       </c>
       <c r="D225" s="4">
-        <v>100000</v>
+        <v>0</v>
       </c>
       <c r="E225" s="4">
-        <v>100000</v>
+        <v>0</v>
       </c>
       <c r="F225" s="4">
-        <v>200000</v>
+        <v>1</v>
       </c>
       <c r="G225" s="4">
-        <v>100000</v>
+        <v>0</v>
       </c>
       <c r="H225" s="4">
-        <v>100000</v>
+        <v>0</v>
       </c>
       <c r="I225" s="4">
-        <v>100000</v>
+        <v>1</v>
       </c>
       <c r="J225" s="4">
-        <v>200000</v>
+        <v>0</v>
       </c>
       <c r="K225" s="4">
-        <v>200000</v>
+        <v>0</v>
       </c>
       <c r="L225" s="4">
-        <v>200000</v>
+        <v>1</v>
       </c>
       <c r="M225" s="4">
-        <v>200000</v>
+        <v>0</v>
       </c>
       <c r="N225" s="4">
-        <v>100000</v>
+        <v>0</v>
       </c>
       <c r="O225" s="4">
-        <v>100000</v>
+        <v>1</v>
       </c>
       <c r="P225" s="4">
-        <v>1700000</v>
+        <v>4</v>
       </c>
       <c r="Q225" s="4" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="R225" s="4" t="s">
         <v>21</v>
@@ -13113,55 +13254,55 @@
     </row>
     <row r="226" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A226" s="4">
-        <v>270035</v>
+        <v>270029</v>
       </c>
       <c r="B226" s="4" t="s">
         <v>75</v>
       </c>
       <c r="C226" s="4" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="D226" s="4">
-        <v>0</v>
+        <v>100000</v>
       </c>
       <c r="E226" s="4">
-        <v>1</v>
+        <v>100000</v>
       </c>
       <c r="F226" s="4">
-        <v>0</v>
+        <v>200000</v>
       </c>
       <c r="G226" s="4">
-        <v>1</v>
+        <v>100000</v>
       </c>
       <c r="H226" s="4">
-        <v>0</v>
+        <v>100000</v>
       </c>
       <c r="I226" s="4">
-        <v>1</v>
+        <v>100000</v>
       </c>
       <c r="J226" s="4">
-        <v>0</v>
+        <v>200000</v>
       </c>
       <c r="K226" s="4">
-        <v>1</v>
+        <v>200000</v>
       </c>
       <c r="L226" s="4">
-        <v>0</v>
+        <v>200000</v>
       </c>
       <c r="M226" s="4">
-        <v>1</v>
+        <v>200000</v>
       </c>
       <c r="N226" s="4">
-        <v>0</v>
+        <v>100000</v>
       </c>
       <c r="O226" s="4">
-        <v>1</v>
+        <v>100000</v>
       </c>
       <c r="P226" s="4">
-        <v>6</v>
+        <v>1700000</v>
       </c>
       <c r="Q226" s="4" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="R226" s="4" t="s">
         <v>21</v>
@@ -13169,13 +13310,13 @@
     </row>
     <row r="227" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A227" s="4">
-        <v>270035</v>
+        <v>270029</v>
       </c>
       <c r="B227" s="4" t="s">
         <v>75</v>
       </c>
       <c r="C227" s="4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D227" s="4">
         <v>0</v>
@@ -13217,7 +13358,7 @@
         <v>6</v>
       </c>
       <c r="Q227" s="4" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="R227" s="4" t="s">
         <v>21</v>
@@ -13225,55 +13366,55 @@
     </row>
     <row r="228" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A228" s="4">
-        <v>270035</v>
+        <v>270029</v>
       </c>
       <c r="B228" s="4" t="s">
         <v>75</v>
       </c>
       <c r="C228" s="4" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="D228" s="4">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E228" s="4">
         <v>1</v>
       </c>
       <c r="F228" s="4">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G228" s="4">
         <v>1</v>
       </c>
       <c r="H228" s="4">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I228" s="4">
         <v>1</v>
       </c>
       <c r="J228" s="4">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K228" s="4">
         <v>1</v>
       </c>
       <c r="L228" s="4">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="M228" s="4">
         <v>1</v>
       </c>
       <c r="N228" s="4">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O228" s="4">
         <v>1</v>
       </c>
       <c r="P228" s="4">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="Q228" s="4" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="R228" s="4" t="s">
         <v>21</v>
@@ -13281,55 +13422,55 @@
     </row>
     <row r="229" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A229" s="4">
-        <v>270035</v>
+        <v>270029</v>
       </c>
       <c r="B229" s="4" t="s">
         <v>75</v>
       </c>
       <c r="C229" s="4" t="s">
-        <v>39</v>
+        <v>28</v>
       </c>
       <c r="D229" s="4">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E229" s="4">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F229" s="4">
         <v>1</v>
       </c>
       <c r="G229" s="4">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H229" s="4">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I229" s="4">
         <v>1</v>
       </c>
       <c r="J229" s="4">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K229" s="4">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L229" s="4">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M229" s="4">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N229" s="4">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O229" s="4">
         <v>1</v>
       </c>
       <c r="P229" s="4">
-        <v>4</v>
+        <v>13</v>
       </c>
       <c r="Q229" s="4" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="R229" s="4" t="s">
         <v>21</v>
@@ -13340,52 +13481,52 @@
         <v>270029</v>
       </c>
       <c r="B230" s="4" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C230" s="4" t="s">
-        <v>19</v>
+        <v>39</v>
       </c>
       <c r="D230" s="4">
-        <v>100000</v>
+        <v>0</v>
       </c>
       <c r="E230" s="4">
-        <v>100000</v>
+        <v>0</v>
       </c>
       <c r="F230" s="4">
-        <v>200000</v>
+        <v>1</v>
       </c>
       <c r="G230" s="4">
-        <v>100000</v>
+        <v>0</v>
       </c>
       <c r="H230" s="4">
-        <v>100000</v>
+        <v>0</v>
       </c>
       <c r="I230" s="4">
-        <v>100000</v>
+        <v>1</v>
       </c>
       <c r="J230" s="4">
-        <v>200000</v>
+        <v>0</v>
       </c>
       <c r="K230" s="4">
-        <v>200000</v>
+        <v>0</v>
       </c>
       <c r="L230" s="4">
-        <v>200000</v>
+        <v>1</v>
       </c>
       <c r="M230" s="4">
-        <v>200000</v>
+        <v>0</v>
       </c>
       <c r="N230" s="4">
-        <v>100000</v>
+        <v>0</v>
       </c>
       <c r="O230" s="4">
-        <v>100000</v>
+        <v>1</v>
       </c>
       <c r="P230" s="4">
-        <v>1700000</v>
+        <v>4</v>
       </c>
       <c r="Q230" s="4" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="R230" s="4" t="s">
         <v>21</v>
@@ -13393,22 +13534,22 @@
     </row>
     <row r="231" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A231" s="4">
-        <v>270029</v>
+        <v>212910</v>
       </c>
       <c r="B231" s="4" t="s">
         <v>76</v>
       </c>
       <c r="C231" s="4" t="s">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="D231" s="4">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E231" s="4">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="F231" s="4">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G231" s="4">
         <v>1</v>
@@ -13420,28 +13561,28 @@
         <v>1</v>
       </c>
       <c r="J231" s="4">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K231" s="4">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L231" s="4">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M231" s="4">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N231" s="4">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O231" s="4">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P231" s="4">
-        <v>6</v>
+        <v>17</v>
       </c>
       <c r="Q231" s="4" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="R231" s="4" t="s">
         <v>21</v>
@@ -13449,55 +13590,55 @@
     </row>
     <row r="232" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A232" s="4">
-        <v>270029</v>
+        <v>212910</v>
       </c>
       <c r="B232" s="4" t="s">
         <v>76</v>
       </c>
       <c r="C232" s="4" t="s">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="D232" s="4">
-        <v>0</v>
+        <v>133333</v>
       </c>
       <c r="E232" s="4">
-        <v>1</v>
+        <v>315152</v>
       </c>
       <c r="F232" s="4">
-        <v>0</v>
+        <v>60606</v>
       </c>
       <c r="G232" s="4">
-        <v>1</v>
+        <v>109091</v>
       </c>
       <c r="H232" s="4">
-        <v>0</v>
+        <v>169697</v>
       </c>
       <c r="I232" s="4">
-        <v>1</v>
+        <v>157576</v>
       </c>
       <c r="J232" s="4">
-        <v>0</v>
+        <v>181818</v>
       </c>
       <c r="K232" s="4">
-        <v>1</v>
+        <v>254545</v>
       </c>
       <c r="L232" s="4">
-        <v>0</v>
+        <v>230303</v>
       </c>
       <c r="M232" s="4">
-        <v>1</v>
+        <v>193939</v>
       </c>
       <c r="N232" s="4">
-        <v>0</v>
+        <v>121213</v>
       </c>
       <c r="O232" s="4">
-        <v>1</v>
+        <v>72727</v>
       </c>
       <c r="P232" s="4">
-        <v>6</v>
+        <v>2000000</v>
       </c>
       <c r="Q232" s="4" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="R232" s="4" t="s">
         <v>21</v>
@@ -13505,55 +13646,55 @@
     </row>
     <row r="233" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A233" s="4">
-        <v>270029</v>
+        <v>212910</v>
       </c>
       <c r="B233" s="4" t="s">
         <v>76</v>
       </c>
       <c r="C233" s="4" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="D233" s="4">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E233" s="4">
         <v>1</v>
       </c>
       <c r="F233" s="4">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G233" s="4">
         <v>1</v>
       </c>
       <c r="H233" s="4">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I233" s="4">
         <v>1</v>
       </c>
       <c r="J233" s="4">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K233" s="4">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L233" s="4">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="M233" s="4">
         <v>1</v>
       </c>
       <c r="N233" s="4">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O233" s="4">
         <v>1</v>
       </c>
       <c r="P233" s="4">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="Q233" s="4" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="R233" s="4" t="s">
         <v>21</v>
@@ -13561,55 +13702,55 @@
     </row>
     <row r="234" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A234" s="4">
-        <v>270029</v>
+        <v>212876</v>
       </c>
       <c r="B234" s="4" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="C234" s="4" t="s">
-        <v>39</v>
+        <v>28</v>
       </c>
       <c r="D234" s="4">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="E234" s="4">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F234" s="4">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G234" s="4">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H234" s="4">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I234" s="4">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="J234" s="4">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="K234" s="4">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="L234" s="4">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M234" s="4">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="N234" s="4">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="O234" s="4">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="P234" s="4">
-        <v>4</v>
+        <v>38</v>
       </c>
       <c r="Q234" s="4" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="R234" s="4" t="s">
         <v>21</v>
@@ -13617,55 +13758,55 @@
     </row>
     <row r="235" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A235" s="4">
-        <v>212910</v>
+        <v>212876</v>
       </c>
       <c r="B235" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="C235" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="D235" s="4">
+        <v>222222</v>
+      </c>
+      <c r="E235" s="4">
+        <v>130719</v>
+      </c>
+      <c r="F235" s="4">
+        <v>222222</v>
+      </c>
+      <c r="G235" s="4">
+        <v>156863</v>
+      </c>
+      <c r="H235" s="4">
+        <v>222222</v>
+      </c>
+      <c r="I235" s="4">
+        <v>91503</v>
+      </c>
+      <c r="J235" s="4">
+        <v>209150</v>
+      </c>
+      <c r="K235" s="4">
+        <v>261438</v>
+      </c>
+      <c r="L235" s="4">
+        <v>143791</v>
+      </c>
+      <c r="M235" s="4">
+        <v>91504</v>
+      </c>
+      <c r="N235" s="4">
+        <v>143791</v>
+      </c>
+      <c r="O235" s="4">
+        <v>104575</v>
+      </c>
+      <c r="P235" s="4">
+        <v>2000000</v>
+      </c>
+      <c r="Q235" s="4" t="s">
         <v>77</v>
-      </c>
-      <c r="C235" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="D235" s="4">
-        <v>1</v>
-      </c>
-      <c r="E235" s="4">
-        <v>5</v>
-      </c>
-      <c r="F235" s="4">
-        <v>1</v>
-      </c>
-      <c r="G235" s="4">
-        <v>1</v>
-      </c>
-      <c r="H235" s="4">
-        <v>0</v>
-      </c>
-      <c r="I235" s="4">
-        <v>1</v>
-      </c>
-      <c r="J235" s="4">
-        <v>2</v>
-      </c>
-      <c r="K235" s="4">
-        <v>2</v>
-      </c>
-      <c r="L235" s="4">
-        <v>1</v>
-      </c>
-      <c r="M235" s="4">
-        <v>2</v>
-      </c>
-      <c r="N235" s="4">
-        <v>1</v>
-      </c>
-      <c r="O235" s="4">
-        <v>0</v>
-      </c>
-      <c r="P235" s="4">
-        <v>17</v>
-      </c>
-      <c r="Q235" s="4" t="s">
-        <v>78</v>
       </c>
       <c r="R235" s="4" t="s">
         <v>21</v>
@@ -13673,281 +13814,57 @@
     </row>
     <row r="236" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A236" s="4">
-        <v>212910</v>
+        <v>212876</v>
       </c>
       <c r="B236" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="C236" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="D236" s="4">
+        <v>0</v>
+      </c>
+      <c r="E236" s="4">
+        <v>1</v>
+      </c>
+      <c r="F236" s="4">
+        <v>0</v>
+      </c>
+      <c r="G236" s="4">
+        <v>1</v>
+      </c>
+      <c r="H236" s="4">
+        <v>0</v>
+      </c>
+      <c r="I236" s="4">
+        <v>1</v>
+      </c>
+      <c r="J236" s="4">
+        <v>0</v>
+      </c>
+      <c r="K236" s="4">
+        <v>0</v>
+      </c>
+      <c r="L236" s="4">
+        <v>0</v>
+      </c>
+      <c r="M236" s="4">
+        <v>1</v>
+      </c>
+      <c r="N236" s="4">
+        <v>0</v>
+      </c>
+      <c r="O236" s="4">
+        <v>1</v>
+      </c>
+      <c r="P236" s="4">
+        <v>5</v>
+      </c>
+      <c r="Q236" s="4" t="s">
         <v>77</v>
       </c>
-      <c r="C236" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="D236" s="4">
-        <v>133333</v>
-      </c>
-      <c r="E236" s="4">
-        <v>315152</v>
-      </c>
-      <c r="F236" s="4">
-        <v>60606</v>
-      </c>
-      <c r="G236" s="4">
-        <v>109091</v>
-      </c>
-      <c r="H236" s="4">
-        <v>169697</v>
-      </c>
-      <c r="I236" s="4">
-        <v>157576</v>
-      </c>
-      <c r="J236" s="4">
-        <v>181818</v>
-      </c>
-      <c r="K236" s="4">
-        <v>254545</v>
-      </c>
-      <c r="L236" s="4">
-        <v>230303</v>
-      </c>
-      <c r="M236" s="4">
-        <v>193939</v>
-      </c>
-      <c r="N236" s="4">
-        <v>121213</v>
-      </c>
-      <c r="O236" s="4">
-        <v>72727</v>
-      </c>
-      <c r="P236" s="4">
-        <v>2000000</v>
-      </c>
-      <c r="Q236" s="4" t="s">
-        <v>78</v>
-      </c>
       <c r="R236" s="4" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="237" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A237" s="4">
-        <v>212910</v>
-      </c>
-      <c r="B237" s="4" t="s">
-        <v>77</v>
-      </c>
-      <c r="C237" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="D237" s="4">
-        <v>0</v>
-      </c>
-      <c r="E237" s="4">
-        <v>1</v>
-      </c>
-      <c r="F237" s="4">
-        <v>0</v>
-      </c>
-      <c r="G237" s="4">
-        <v>1</v>
-      </c>
-      <c r="H237" s="4">
-        <v>0</v>
-      </c>
-      <c r="I237" s="4">
-        <v>1</v>
-      </c>
-      <c r="J237" s="4">
-        <v>0</v>
-      </c>
-      <c r="K237" s="4">
-        <v>0</v>
-      </c>
-      <c r="L237" s="4">
-        <v>0</v>
-      </c>
-      <c r="M237" s="4">
-        <v>1</v>
-      </c>
-      <c r="N237" s="4">
-        <v>0</v>
-      </c>
-      <c r="O237" s="4">
-        <v>1</v>
-      </c>
-      <c r="P237" s="4">
-        <v>5</v>
-      </c>
-      <c r="Q237" s="4" t="s">
-        <v>78</v>
-      </c>
-      <c r="R237" s="4" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="238" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A238" s="4">
-        <v>212876</v>
-      </c>
-      <c r="B238" s="4" t="s">
-        <v>79</v>
-      </c>
-      <c r="C238" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="D238" s="4">
-        <v>4</v>
-      </c>
-      <c r="E238" s="4">
-        <v>3</v>
-      </c>
-      <c r="F238" s="4">
-        <v>3</v>
-      </c>
-      <c r="G238" s="4">
-        <v>3</v>
-      </c>
-      <c r="H238" s="4">
-        <v>2</v>
-      </c>
-      <c r="I238" s="4">
-        <v>4</v>
-      </c>
-      <c r="J238" s="4">
-        <v>4</v>
-      </c>
-      <c r="K238" s="4">
-        <v>4</v>
-      </c>
-      <c r="L238" s="4">
-        <v>2</v>
-      </c>
-      <c r="M238" s="4">
-        <v>3</v>
-      </c>
-      <c r="N238" s="4">
-        <v>3</v>
-      </c>
-      <c r="O238" s="4">
-        <v>3</v>
-      </c>
-      <c r="P238" s="4">
-        <v>38</v>
-      </c>
-      <c r="Q238" s="4" t="s">
-        <v>78</v>
-      </c>
-      <c r="R238" s="4" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="239" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A239" s="4">
-        <v>212876</v>
-      </c>
-      <c r="B239" s="4" t="s">
-        <v>79</v>
-      </c>
-      <c r="C239" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="D239" s="4">
-        <v>222222</v>
-      </c>
-      <c r="E239" s="4">
-        <v>130719</v>
-      </c>
-      <c r="F239" s="4">
-        <v>222222</v>
-      </c>
-      <c r="G239" s="4">
-        <v>156863</v>
-      </c>
-      <c r="H239" s="4">
-        <v>222222</v>
-      </c>
-      <c r="I239" s="4">
-        <v>91503</v>
-      </c>
-      <c r="J239" s="4">
-        <v>209150</v>
-      </c>
-      <c r="K239" s="4">
-        <v>261438</v>
-      </c>
-      <c r="L239" s="4">
-        <v>143791</v>
-      </c>
-      <c r="M239" s="4">
-        <v>91504</v>
-      </c>
-      <c r="N239" s="4">
-        <v>143791</v>
-      </c>
-      <c r="O239" s="4">
-        <v>104575</v>
-      </c>
-      <c r="P239" s="4">
-        <v>2000000</v>
-      </c>
-      <c r="Q239" s="4" t="s">
-        <v>78</v>
-      </c>
-      <c r="R239" s="4" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="240" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A240" s="4">
-        <v>212876</v>
-      </c>
-      <c r="B240" s="4" t="s">
-        <v>79</v>
-      </c>
-      <c r="C240" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="D240" s="4">
-        <v>0</v>
-      </c>
-      <c r="E240" s="4">
-        <v>1</v>
-      </c>
-      <c r="F240" s="4">
-        <v>0</v>
-      </c>
-      <c r="G240" s="4">
-        <v>1</v>
-      </c>
-      <c r="H240" s="4">
-        <v>0</v>
-      </c>
-      <c r="I240" s="4">
-        <v>1</v>
-      </c>
-      <c r="J240" s="4">
-        <v>0</v>
-      </c>
-      <c r="K240" s="4">
-        <v>0</v>
-      </c>
-      <c r="L240" s="4">
-        <v>0</v>
-      </c>
-      <c r="M240" s="4">
-        <v>1</v>
-      </c>
-      <c r="N240" s="4">
-        <v>0</v>
-      </c>
-      <c r="O240" s="4">
-        <v>1</v>
-      </c>
-      <c r="P240" s="4">
-        <v>5</v>
-      </c>
-      <c r="Q240" s="4" t="s">
-        <v>78</v>
-      </c>
-      <c r="R240" s="4" t="s">
         <v>21</v>
       </c>
     </row>
@@ -13966,17 +13883,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="f76aa77c-8923-4724-9a6d-d588cc513697">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="89c54d5b-05ac-45d5-9242-aabb385cc5ad" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100B96036E30F13644F923D207E371C305D" ma:contentTypeVersion="11" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="1d197ceb99055fd1a93a3a14aec1bdd8">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="f76aa77c-8923-4724-9a6d-d588cc513697" xmlns:ns3="89c54d5b-05ac-45d5-9242-aabb385cc5ad" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="5b86266bfd619f312673123d0bd20d23" ns2:_="" ns3:_="">
     <xsd:import namespace="f76aa77c-8923-4724-9a6d-d588cc513697"/>
@@ -14171,6 +14077,17 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="f76aa77c-8923-4724-9a6d-d588cc513697">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="89c54d5b-05ac-45d5-9242-aabb385cc5ad" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F5CFE981-CBAC-4360-B0CE-AB3235A33930}">
   <ds:schemaRefs>
@@ -14180,23 +14097,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F919D1BA-3E11-4877-AEE4-5A5340B7B50A}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="89c54d5b-05ac-45d5-9242-aabb385cc5ad"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="f76aa77c-8923-4724-9a6d-d588cc513697"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8BDC8EFC-C946-4B3C-B84E-1270F018751C}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -14213,4 +14113,21 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F919D1BA-3E11-4877-AEE4-5A5340B7B50A}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="89c54d5b-05ac-45d5-9242-aabb385cc5ad"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="f76aa77c-8923-4724-9a6d-d588cc513697"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Add Orçamento view for Loja tab (Toggle 2)
When Loja + Orçamento selected, loads from ORÇAMENTO sheet in metas.xlsx.
Shared helper _normalizar_sheet_loja() avoids code duplication between
LOJA and ORÇAMENTO loaders.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/dados/metas.xlsx
+++ b/dados/metas.xlsx
@@ -8,13 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pedro.sa\Documents\dashboard-oportunidades\dados\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{96DE449A-755E-477D-985A-0F21147DD0A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF6F0D15-0D99-4E6B-B61C-EE6A713768C5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="CONSULTOR" sheetId="1" r:id="rId1"/>
     <sheet name="LOJA" sheetId="2" r:id="rId2"/>
+    <sheet name="ORÇAMENTO" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">CONSULTOR!$A$1:$R$236</definedName>
@@ -40,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1212" uniqueCount="92">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1466" uniqueCount="92">
   <si>
     <t>CÓD</t>
   </si>
@@ -363,12 +364,18 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="3">
@@ -435,10 +442,10 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -16033,562 +16040,562 @@
       </c>
     </row>
     <row r="38" spans="1:18" ht="18" x14ac:dyDescent="0.25">
-      <c r="A38" s="9">
+      <c r="A38" s="5">
         <v>17</v>
       </c>
-      <c r="B38" s="9" t="s">
+      <c r="B38" s="5" t="s">
         <v>89</v>
       </c>
-      <c r="C38" s="9" t="s">
+      <c r="C38" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="D38" s="9">
+      <c r="D38" s="5">
         <v>6</v>
       </c>
-      <c r="E38" s="9">
+      <c r="E38" s="5">
         <v>8</v>
       </c>
-      <c r="F38" s="9">
+      <c r="F38" s="5">
         <v>8</v>
       </c>
-      <c r="G38" s="9">
+      <c r="G38" s="5">
         <v>7</v>
       </c>
-      <c r="H38" s="9">
+      <c r="H38" s="5">
         <v>7</v>
       </c>
-      <c r="I38" s="9">
+      <c r="I38" s="5">
         <v>8</v>
       </c>
-      <c r="J38" s="9">
+      <c r="J38" s="5">
         <v>8</v>
       </c>
-      <c r="K38" s="9">
+      <c r="K38" s="5">
         <v>10</v>
       </c>
-      <c r="L38" s="9">
+      <c r="L38" s="5">
         <v>10</v>
       </c>
-      <c r="M38" s="9">
+      <c r="M38" s="5">
         <v>11</v>
       </c>
-      <c r="N38" s="9">
+      <c r="N38" s="5">
         <v>7</v>
       </c>
-      <c r="O38" s="9">
+      <c r="O38" s="5">
         <v>7</v>
       </c>
-      <c r="P38" s="10">
+      <c r="P38" s="6">
         <v>97</v>
       </c>
-      <c r="Q38" s="9" t="s">
+      <c r="Q38" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="R38" s="9" t="s">
+      <c r="R38" s="5" t="s">
         <v>88</v>
       </c>
     </row>
     <row r="39" spans="1:18" ht="18" x14ac:dyDescent="0.25">
-      <c r="A39" s="9">
+      <c r="A39" s="5">
         <v>17</v>
       </c>
-      <c r="B39" s="9" t="s">
+      <c r="B39" s="5" t="s">
         <v>89</v>
       </c>
-      <c r="C39" s="9" t="s">
+      <c r="C39" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="D39" s="9">
-        <v>0</v>
-      </c>
-      <c r="E39" s="9">
-        <v>1</v>
-      </c>
-      <c r="F39" s="9">
+      <c r="D39" s="5">
+        <v>0</v>
+      </c>
+      <c r="E39" s="5">
+        <v>1</v>
+      </c>
+      <c r="F39" s="5">
         <v>2</v>
       </c>
-      <c r="G39" s="9">
-        <v>0</v>
-      </c>
-      <c r="H39" s="9">
+      <c r="G39" s="5">
+        <v>0</v>
+      </c>
+      <c r="H39" s="5">
         <v>2</v>
       </c>
-      <c r="I39" s="9">
-        <v>0</v>
-      </c>
-      <c r="J39" s="9">
-        <v>0</v>
-      </c>
-      <c r="K39" s="9">
+      <c r="I39" s="5">
+        <v>0</v>
+      </c>
+      <c r="J39" s="5">
+        <v>0</v>
+      </c>
+      <c r="K39" s="5">
         <v>4</v>
       </c>
-      <c r="L39" s="9">
-        <v>0</v>
-      </c>
-      <c r="M39" s="9">
-        <v>0</v>
-      </c>
-      <c r="N39" s="9">
-        <v>1</v>
-      </c>
-      <c r="O39" s="9">
-        <v>0</v>
-      </c>
-      <c r="P39" s="10">
+      <c r="L39" s="5">
+        <v>0</v>
+      </c>
+      <c r="M39" s="5">
+        <v>0</v>
+      </c>
+      <c r="N39" s="5">
+        <v>1</v>
+      </c>
+      <c r="O39" s="5">
+        <v>0</v>
+      </c>
+      <c r="P39" s="6">
         <v>9</v>
       </c>
-      <c r="Q39" s="9" t="s">
+      <c r="Q39" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="R39" s="9" t="s">
+      <c r="R39" s="5" t="s">
         <v>88</v>
       </c>
     </row>
     <row r="40" spans="1:18" ht="18" x14ac:dyDescent="0.25">
-      <c r="A40" s="9">
+      <c r="A40" s="5">
         <v>17</v>
       </c>
-      <c r="B40" s="9" t="s">
+      <c r="B40" s="5" t="s">
         <v>89</v>
       </c>
-      <c r="C40" s="9" t="s">
+      <c r="C40" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="D40" s="9">
+      <c r="D40" s="5">
         <v>2</v>
       </c>
-      <c r="E40" s="9">
+      <c r="E40" s="5">
         <v>6</v>
       </c>
-      <c r="F40" s="9">
-        <v>1</v>
-      </c>
-      <c r="G40" s="9">
-        <v>0</v>
-      </c>
-      <c r="H40" s="9">
-        <v>0</v>
-      </c>
-      <c r="I40" s="9">
+      <c r="F40" s="5">
+        <v>1</v>
+      </c>
+      <c r="G40" s="5">
+        <v>0</v>
+      </c>
+      <c r="H40" s="5">
+        <v>0</v>
+      </c>
+      <c r="I40" s="5">
         <v>2</v>
       </c>
-      <c r="J40" s="9">
-        <v>0</v>
-      </c>
-      <c r="K40" s="9">
+      <c r="J40" s="5">
+        <v>0</v>
+      </c>
+      <c r="K40" s="5">
         <v>3</v>
       </c>
-      <c r="L40" s="9">
+      <c r="L40" s="5">
         <v>4</v>
       </c>
-      <c r="M40" s="9">
+      <c r="M40" s="5">
         <v>4</v>
       </c>
-      <c r="N40" s="9">
+      <c r="N40" s="5">
         <v>2</v>
       </c>
-      <c r="O40" s="9">
+      <c r="O40" s="5">
         <v>2</v>
       </c>
-      <c r="P40" s="10">
+      <c r="P40" s="6">
         <v>29</v>
       </c>
-      <c r="Q40" s="9" t="s">
+      <c r="Q40" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="R40" s="9" t="s">
+      <c r="R40" s="5" t="s">
         <v>88</v>
       </c>
     </row>
     <row r="41" spans="1:18" ht="18" x14ac:dyDescent="0.25">
-      <c r="A41" s="9">
+      <c r="A41" s="5">
         <v>17</v>
       </c>
-      <c r="B41" s="9" t="s">
+      <c r="B41" s="5" t="s">
         <v>89</v>
       </c>
-      <c r="C41" s="9" t="s">
+      <c r="C41" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="D41" s="9">
-        <v>0</v>
-      </c>
-      <c r="E41" s="9">
+      <c r="D41" s="5">
+        <v>0</v>
+      </c>
+      <c r="E41" s="5">
         <v>2</v>
       </c>
-      <c r="F41" s="9">
-        <v>0</v>
-      </c>
-      <c r="G41" s="9">
-        <v>0</v>
-      </c>
-      <c r="H41" s="9">
-        <v>0</v>
-      </c>
-      <c r="I41" s="9">
-        <v>0</v>
-      </c>
-      <c r="J41" s="9">
-        <v>0</v>
-      </c>
-      <c r="K41" s="9">
+      <c r="F41" s="5">
+        <v>0</v>
+      </c>
+      <c r="G41" s="5">
+        <v>0</v>
+      </c>
+      <c r="H41" s="5">
+        <v>0</v>
+      </c>
+      <c r="I41" s="5">
+        <v>0</v>
+      </c>
+      <c r="J41" s="5">
+        <v>0</v>
+      </c>
+      <c r="K41" s="5">
         <v>3</v>
       </c>
-      <c r="L41" s="9">
-        <v>1</v>
-      </c>
-      <c r="M41" s="9">
+      <c r="L41" s="5">
+        <v>1</v>
+      </c>
+      <c r="M41" s="5">
         <v>5</v>
       </c>
-      <c r="N41" s="9">
-        <v>0</v>
-      </c>
-      <c r="O41" s="9">
-        <v>0</v>
-      </c>
-      <c r="P41" s="10">
+      <c r="N41" s="5">
+        <v>0</v>
+      </c>
+      <c r="O41" s="5">
+        <v>0</v>
+      </c>
+      <c r="P41" s="6">
         <v>11</v>
       </c>
-      <c r="Q41" s="9" t="s">
+      <c r="Q41" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="R41" s="9" t="s">
+      <c r="R41" s="5" t="s">
         <v>88</v>
       </c>
     </row>
     <row r="42" spans="1:18" ht="18" x14ac:dyDescent="0.25">
-      <c r="A42" s="9">
+      <c r="A42" s="5">
         <v>17</v>
       </c>
-      <c r="B42" s="9" t="s">
+      <c r="B42" s="5" t="s">
         <v>89</v>
       </c>
-      <c r="C42" s="9" t="s">
+      <c r="C42" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="D42" s="9">
+      <c r="D42" s="5">
         <v>2</v>
       </c>
-      <c r="E42" s="9">
+      <c r="E42" s="5">
         <v>5</v>
       </c>
-      <c r="F42" s="9">
+      <c r="F42" s="5">
         <v>2</v>
       </c>
-      <c r="G42" s="9">
-        <v>0</v>
-      </c>
-      <c r="H42" s="9">
-        <v>0</v>
-      </c>
-      <c r="I42" s="9">
+      <c r="G42" s="5">
+        <v>0</v>
+      </c>
+      <c r="H42" s="5">
+        <v>0</v>
+      </c>
+      <c r="I42" s="5">
         <v>2</v>
       </c>
-      <c r="J42" s="9">
-        <v>0</v>
-      </c>
-      <c r="K42" s="9">
+      <c r="J42" s="5">
+        <v>0</v>
+      </c>
+      <c r="K42" s="5">
         <v>3</v>
       </c>
-      <c r="L42" s="9">
+      <c r="L42" s="5">
         <v>4</v>
       </c>
-      <c r="M42" s="9">
+      <c r="M42" s="5">
         <v>5</v>
       </c>
-      <c r="N42" s="9">
+      <c r="N42" s="5">
         <v>2</v>
       </c>
-      <c r="O42" s="9">
+      <c r="O42" s="5">
         <v>2</v>
       </c>
-      <c r="P42" s="10">
+      <c r="P42" s="6">
         <v>29</v>
       </c>
-      <c r="Q42" s="9" t="s">
+      <c r="Q42" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="R42" s="9" t="s">
+      <c r="R42" s="5" t="s">
         <v>88</v>
       </c>
     </row>
     <row r="43" spans="1:18" ht="18" x14ac:dyDescent="0.25">
-      <c r="A43" s="9">
+      <c r="A43" s="5">
         <v>17</v>
       </c>
-      <c r="B43" s="9" t="s">
+      <c r="B43" s="5" t="s">
         <v>89</v>
       </c>
-      <c r="C43" s="9" t="s">
+      <c r="C43" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="D43" s="9">
-        <v>0</v>
-      </c>
-      <c r="E43" s="9">
+      <c r="D43" s="5">
+        <v>0</v>
+      </c>
+      <c r="E43" s="5">
         <v>6</v>
       </c>
-      <c r="F43" s="9">
-        <v>1</v>
-      </c>
-      <c r="G43" s="9">
-        <v>0</v>
-      </c>
-      <c r="H43" s="9">
+      <c r="F43" s="5">
+        <v>1</v>
+      </c>
+      <c r="G43" s="5">
+        <v>0</v>
+      </c>
+      <c r="H43" s="5">
         <v>4</v>
       </c>
-      <c r="I43" s="9">
-        <v>0</v>
-      </c>
-      <c r="J43" s="9">
+      <c r="I43" s="5">
+        <v>0</v>
+      </c>
+      <c r="J43" s="5">
         <v>4</v>
       </c>
-      <c r="K43" s="9">
+      <c r="K43" s="5">
         <v>5</v>
       </c>
-      <c r="L43" s="9">
-        <v>0</v>
-      </c>
-      <c r="M43" s="9">
-        <v>0</v>
-      </c>
-      <c r="N43" s="9">
-        <v>1</v>
-      </c>
-      <c r="O43" s="9">
-        <v>0</v>
-      </c>
-      <c r="P43" s="10">
+      <c r="L43" s="5">
+        <v>0</v>
+      </c>
+      <c r="M43" s="5">
+        <v>0</v>
+      </c>
+      <c r="N43" s="5">
+        <v>1</v>
+      </c>
+      <c r="O43" s="5">
+        <v>0</v>
+      </c>
+      <c r="P43" s="6">
         <v>24</v>
       </c>
-      <c r="Q43" s="9" t="s">
+      <c r="Q43" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="R43" s="9" t="s">
+      <c r="R43" s="5" t="s">
         <v>88</v>
       </c>
     </row>
     <row r="44" spans="1:18" ht="18" x14ac:dyDescent="0.25">
-      <c r="A44" s="9">
+      <c r="A44" s="5">
         <v>17</v>
       </c>
-      <c r="B44" s="9" t="s">
+      <c r="B44" s="5" t="s">
         <v>89</v>
       </c>
-      <c r="C44" s="9" t="s">
+      <c r="C44" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="D44" s="9">
+      <c r="D44" s="5">
         <v>891473</v>
       </c>
-      <c r="E44" s="9">
+      <c r="E44" s="5">
         <v>1472867</v>
       </c>
-      <c r="F44" s="9">
+      <c r="F44" s="5">
         <v>1395350</v>
       </c>
-      <c r="G44" s="9">
+      <c r="G44" s="5">
         <v>838501</v>
       </c>
-      <c r="H44" s="9">
+      <c r="H44" s="5">
         <v>740051</v>
       </c>
-      <c r="I44" s="9">
+      <c r="I44" s="5">
         <v>1023256</v>
       </c>
-      <c r="J44" s="9">
+      <c r="J44" s="5">
         <v>1380620</v>
       </c>
-      <c r="K44" s="9">
+      <c r="K44" s="5">
         <v>1321706</v>
       </c>
-      <c r="L44" s="9">
+      <c r="L44" s="5">
         <v>1294315</v>
       </c>
-      <c r="M44" s="9">
+      <c r="M44" s="5">
         <v>1136951</v>
       </c>
-      <c r="N44" s="9">
+      <c r="N44" s="5">
         <v>1125323</v>
       </c>
-      <c r="O44" s="9">
+      <c r="O44" s="5">
         <v>882171</v>
       </c>
-      <c r="P44" s="10">
+      <c r="P44" s="6">
         <v>15000000</v>
       </c>
-      <c r="Q44" s="9" t="s">
+      <c r="Q44" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="R44" s="9" t="s">
+      <c r="R44" s="5" t="s">
         <v>88</v>
       </c>
     </row>
     <row r="45" spans="1:18" ht="18" x14ac:dyDescent="0.25">
-      <c r="A45" s="9">
+      <c r="A45" s="5">
         <v>17</v>
       </c>
-      <c r="B45" s="9" t="s">
+      <c r="B45" s="5" t="s">
         <v>89</v>
       </c>
-      <c r="C45" s="9" t="s">
+      <c r="C45" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="D45" s="9">
+      <c r="D45" s="5">
         <v>576486</v>
       </c>
-      <c r="E45" s="9">
+      <c r="E45" s="5">
         <v>952455</v>
       </c>
-      <c r="F45" s="9">
+      <c r="F45" s="5">
         <v>902326</v>
       </c>
-      <c r="G45" s="9">
+      <c r="G45" s="5">
         <v>656952</v>
       </c>
-      <c r="H45" s="9">
+      <c r="H45" s="5">
         <v>448036</v>
       </c>
-      <c r="I45" s="9">
+      <c r="I45" s="5">
         <v>806280</v>
       </c>
-      <c r="J45" s="9">
+      <c r="J45" s="5">
         <v>776434</v>
       </c>
-      <c r="K45" s="9">
+      <c r="K45" s="5">
         <v>1045195</v>
       </c>
-      <c r="L45" s="9">
+      <c r="L45" s="5">
         <v>866021</v>
       </c>
-      <c r="M45" s="9">
+      <c r="M45" s="5">
         <v>915865</v>
       </c>
-      <c r="N45" s="9">
+      <c r="N45" s="5">
         <v>507726</v>
       </c>
-      <c r="O45" s="9">
+      <c r="O45" s="5">
         <v>547520</v>
       </c>
-      <c r="P45" s="10">
+      <c r="P45" s="6">
         <v>9700004</v>
       </c>
-      <c r="Q45" s="9" t="s">
+      <c r="Q45" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="R45" s="9" t="s">
+      <c r="R45" s="5" t="s">
         <v>88</v>
       </c>
     </row>
     <row r="46" spans="1:18" ht="18" x14ac:dyDescent="0.25">
-      <c r="A46" s="9">
+      <c r="A46" s="5">
         <v>17</v>
       </c>
-      <c r="B46" s="9" t="s">
+      <c r="B46" s="5" t="s">
         <v>89</v>
       </c>
-      <c r="C46" s="9" t="s">
+      <c r="C46" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="D46" s="9">
-        <v>0</v>
-      </c>
-      <c r="E46" s="9">
+      <c r="D46" s="5">
+        <v>0</v>
+      </c>
+      <c r="E46" s="5">
         <v>6</v>
       </c>
-      <c r="F46" s="9">
-        <v>0</v>
-      </c>
-      <c r="G46" s="9">
-        <v>0</v>
-      </c>
-      <c r="H46" s="9">
+      <c r="F46" s="5">
+        <v>0</v>
+      </c>
+      <c r="G46" s="5">
+        <v>0</v>
+      </c>
+      <c r="H46" s="5">
         <v>5</v>
       </c>
-      <c r="I46" s="9">
+      <c r="I46" s="5">
         <v>4</v>
       </c>
-      <c r="J46" s="9">
+      <c r="J46" s="5">
         <v>5</v>
       </c>
-      <c r="K46" s="9">
-        <v>0</v>
-      </c>
-      <c r="L46" s="9">
+      <c r="K46" s="5">
+        <v>0</v>
+      </c>
+      <c r="L46" s="5">
         <v>3</v>
       </c>
-      <c r="M46" s="9">
+      <c r="M46" s="5">
         <v>2</v>
       </c>
-      <c r="N46" s="9">
-        <v>0</v>
-      </c>
-      <c r="O46" s="9">
-        <v>0</v>
-      </c>
-      <c r="P46" s="10">
+      <c r="N46" s="5">
+        <v>0</v>
+      </c>
+      <c r="O46" s="5">
+        <v>0</v>
+      </c>
+      <c r="P46" s="6">
         <v>28</v>
       </c>
-      <c r="Q46" s="9" t="s">
+      <c r="Q46" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="R46" s="9" t="s">
+      <c r="R46" s="5" t="s">
         <v>88</v>
       </c>
     </row>
     <row r="47" spans="1:18" ht="18" x14ac:dyDescent="0.25">
-      <c r="A47" s="9">
+      <c r="A47" s="5">
         <v>17</v>
       </c>
-      <c r="B47" s="9" t="s">
+      <c r="B47" s="5" t="s">
         <v>89</v>
       </c>
-      <c r="C47" s="9" t="s">
+      <c r="C47" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="D47" s="9">
+      <c r="D47" s="5">
         <v>6</v>
       </c>
-      <c r="E47" s="9">
+      <c r="E47" s="5">
         <v>6</v>
       </c>
-      <c r="F47" s="9">
+      <c r="F47" s="5">
         <v>6</v>
       </c>
-      <c r="G47" s="9">
+      <c r="G47" s="5">
         <v>5</v>
       </c>
-      <c r="H47" s="9">
+      <c r="H47" s="5">
         <v>5</v>
       </c>
-      <c r="I47" s="9">
+      <c r="I47" s="5">
         <v>5</v>
       </c>
-      <c r="J47" s="9">
+      <c r="J47" s="5">
         <v>5</v>
       </c>
-      <c r="K47" s="9">
+      <c r="K47" s="5">
         <v>5</v>
       </c>
-      <c r="L47" s="9">
+      <c r="L47" s="5">
         <v>5</v>
       </c>
-      <c r="M47" s="9">
+      <c r="M47" s="5">
         <v>5</v>
       </c>
-      <c r="N47" s="9">
+      <c r="N47" s="5">
         <v>5</v>
       </c>
-      <c r="O47" s="9">
+      <c r="O47" s="5">
         <v>5</v>
       </c>
-      <c r="P47" s="10">
+      <c r="P47" s="6">
         <v>72</v>
       </c>
-      <c r="Q47" s="9" t="s">
+      <c r="Q47" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="R47" s="9" t="s">
+      <c r="R47" s="5" t="s">
         <v>88</v>
       </c>
     </row>
@@ -19645,16 +19652,1848 @@
 </worksheet>
 </file>
 
-<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A764B28F-457A-4F3D-AEF6-E9832275A92C}">
+  <dimension ref="A1:R60"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="4.85546875" customWidth="1"/>
+    <col min="2" max="2" width="16.42578125" customWidth="1"/>
+    <col min="3" max="3" width="14.42578125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="N1" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="O1" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="P1" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="Q1" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="R1" s="3" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="2" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A2" s="9">
+        <v>18</v>
+      </c>
+      <c r="B2" s="9" t="s">
+        <v>81</v>
+      </c>
+      <c r="C2" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="D2" s="9"/>
+      <c r="E2" s="9"/>
+      <c r="F2" s="9"/>
+      <c r="G2" s="9"/>
+      <c r="H2" s="9"/>
+      <c r="I2" s="9"/>
+      <c r="J2" s="9"/>
+      <c r="K2" s="9"/>
+      <c r="L2" s="9"/>
+      <c r="M2" s="9"/>
+      <c r="N2" s="9"/>
+      <c r="O2" s="9"/>
+      <c r="P2" s="10"/>
+      <c r="Q2" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="R2" s="9" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="3" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A3" s="9">
+        <v>18</v>
+      </c>
+      <c r="B3" s="9" t="s">
+        <v>81</v>
+      </c>
+      <c r="C3" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="D3" s="9"/>
+      <c r="E3" s="9"/>
+      <c r="F3" s="9"/>
+      <c r="G3" s="9"/>
+      <c r="H3" s="9"/>
+      <c r="I3" s="9"/>
+      <c r="J3" s="9"/>
+      <c r="K3" s="9"/>
+      <c r="L3" s="9"/>
+      <c r="M3" s="9"/>
+      <c r="N3" s="9"/>
+      <c r="O3" s="9"/>
+      <c r="P3" s="10"/>
+      <c r="Q3" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="R3" s="9" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="4" spans="1:18" ht="18" x14ac:dyDescent="0.25">
+      <c r="A4" s="9">
+        <v>18</v>
+      </c>
+      <c r="B4" s="9" t="s">
+        <v>81</v>
+      </c>
+      <c r="C4" s="9" t="s">
+        <v>39</v>
+      </c>
+      <c r="D4" s="9"/>
+      <c r="E4" s="9"/>
+      <c r="F4" s="9"/>
+      <c r="G4" s="9"/>
+      <c r="H4" s="9"/>
+      <c r="I4" s="9"/>
+      <c r="J4" s="9"/>
+      <c r="K4" s="9"/>
+      <c r="L4" s="9"/>
+      <c r="M4" s="9"/>
+      <c r="N4" s="9"/>
+      <c r="O4" s="9"/>
+      <c r="P4" s="10"/>
+      <c r="Q4" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="R4" s="9" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="5" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A5" s="9">
+        <v>18</v>
+      </c>
+      <c r="B5" s="9" t="s">
+        <v>81</v>
+      </c>
+      <c r="C5" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="D5" s="9"/>
+      <c r="E5" s="9"/>
+      <c r="F5" s="9"/>
+      <c r="G5" s="9"/>
+      <c r="H5" s="9"/>
+      <c r="I5" s="9"/>
+      <c r="J5" s="9"/>
+      <c r="K5" s="9"/>
+      <c r="L5" s="9"/>
+      <c r="M5" s="9"/>
+      <c r="N5" s="9"/>
+      <c r="O5" s="9"/>
+      <c r="P5" s="10"/>
+      <c r="Q5" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="R5" s="9" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="6" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A6" s="9">
+        <v>18</v>
+      </c>
+      <c r="B6" s="9" t="s">
+        <v>81</v>
+      </c>
+      <c r="C6" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="D6" s="9"/>
+      <c r="E6" s="9"/>
+      <c r="F6" s="9"/>
+      <c r="G6" s="9"/>
+      <c r="H6" s="9"/>
+      <c r="I6" s="9"/>
+      <c r="J6" s="9"/>
+      <c r="K6" s="9"/>
+      <c r="L6" s="9"/>
+      <c r="M6" s="9"/>
+      <c r="N6" s="9"/>
+      <c r="O6" s="9"/>
+      <c r="P6" s="10"/>
+      <c r="Q6" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="R6" s="9" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="7" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A7" s="5">
+        <v>10</v>
+      </c>
+      <c r="B7" s="5" t="s">
+        <v>83</v>
+      </c>
+      <c r="C7" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="D7" s="5"/>
+      <c r="E7" s="5"/>
+      <c r="F7" s="5"/>
+      <c r="G7" s="5"/>
+      <c r="H7" s="5"/>
+      <c r="I7" s="5"/>
+      <c r="J7" s="5"/>
+      <c r="K7" s="5"/>
+      <c r="L7" s="5"/>
+      <c r="M7" s="5"/>
+      <c r="N7" s="5"/>
+      <c r="O7" s="5"/>
+      <c r="P7" s="6"/>
+      <c r="Q7" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="R7" s="5" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="8" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A8" s="5">
+        <v>10</v>
+      </c>
+      <c r="B8" s="5" t="s">
+        <v>83</v>
+      </c>
+      <c r="C8" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="D8" s="5"/>
+      <c r="E8" s="5"/>
+      <c r="F8" s="5"/>
+      <c r="G8" s="5"/>
+      <c r="H8" s="5"/>
+      <c r="I8" s="5"/>
+      <c r="J8" s="5"/>
+      <c r="K8" s="5"/>
+      <c r="L8" s="5"/>
+      <c r="M8" s="5"/>
+      <c r="N8" s="5"/>
+      <c r="O8" s="5"/>
+      <c r="P8" s="6"/>
+      <c r="Q8" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="R8" s="5" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="9" spans="1:18" ht="18" x14ac:dyDescent="0.25">
+      <c r="A9" s="5">
+        <v>10</v>
+      </c>
+      <c r="B9" s="5" t="s">
+        <v>83</v>
+      </c>
+      <c r="C9" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="D9" s="5"/>
+      <c r="E9" s="5"/>
+      <c r="F9" s="5"/>
+      <c r="G9" s="5"/>
+      <c r="H9" s="5"/>
+      <c r="I9" s="5"/>
+      <c r="J9" s="5"/>
+      <c r="K9" s="5"/>
+      <c r="L9" s="5"/>
+      <c r="M9" s="5"/>
+      <c r="N9" s="5"/>
+      <c r="O9" s="5"/>
+      <c r="P9" s="6"/>
+      <c r="Q9" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="R9" s="5" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="10" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A10" s="5">
+        <v>10</v>
+      </c>
+      <c r="B10" s="5" t="s">
+        <v>83</v>
+      </c>
+      <c r="C10" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="D10" s="5"/>
+      <c r="E10" s="5"/>
+      <c r="F10" s="5"/>
+      <c r="G10" s="5"/>
+      <c r="H10" s="5"/>
+      <c r="I10" s="5"/>
+      <c r="J10" s="5"/>
+      <c r="K10" s="5"/>
+      <c r="L10" s="5"/>
+      <c r="M10" s="5"/>
+      <c r="N10" s="5"/>
+      <c r="O10" s="5"/>
+      <c r="P10" s="6"/>
+      <c r="Q10" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="R10" s="5" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="11" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A11" s="5">
+        <v>10</v>
+      </c>
+      <c r="B11" s="5" t="s">
+        <v>83</v>
+      </c>
+      <c r="C11" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="D11" s="5"/>
+      <c r="E11" s="5"/>
+      <c r="F11" s="5"/>
+      <c r="G11" s="5"/>
+      <c r="H11" s="5"/>
+      <c r="I11" s="5"/>
+      <c r="J11" s="5"/>
+      <c r="K11" s="5"/>
+      <c r="L11" s="5"/>
+      <c r="M11" s="5"/>
+      <c r="N11" s="5"/>
+      <c r="O11" s="5"/>
+      <c r="P11" s="6"/>
+      <c r="Q11" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="R11" s="5" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="12" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A12" s="9">
+        <v>16</v>
+      </c>
+      <c r="B12" s="9" t="s">
+        <v>84</v>
+      </c>
+      <c r="C12" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="D12" s="9"/>
+      <c r="E12" s="9"/>
+      <c r="F12" s="9"/>
+      <c r="G12" s="9"/>
+      <c r="H12" s="9"/>
+      <c r="I12" s="9"/>
+      <c r="J12" s="9"/>
+      <c r="K12" s="9"/>
+      <c r="L12" s="9"/>
+      <c r="M12" s="9"/>
+      <c r="N12" s="9"/>
+      <c r="O12" s="9"/>
+      <c r="P12" s="10"/>
+      <c r="Q12" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="R12" s="9" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="13" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A13" s="9">
+        <v>16</v>
+      </c>
+      <c r="B13" s="9" t="s">
+        <v>84</v>
+      </c>
+      <c r="C13" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="D13" s="9"/>
+      <c r="E13" s="9"/>
+      <c r="F13" s="9"/>
+      <c r="G13" s="9"/>
+      <c r="H13" s="9"/>
+      <c r="I13" s="9"/>
+      <c r="J13" s="9"/>
+      <c r="K13" s="9"/>
+      <c r="L13" s="9"/>
+      <c r="M13" s="9"/>
+      <c r="N13" s="9"/>
+      <c r="O13" s="9"/>
+      <c r="P13" s="10"/>
+      <c r="Q13" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="R13" s="9" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="14" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A14" s="9">
+        <v>16</v>
+      </c>
+      <c r="B14" s="9" t="s">
+        <v>84</v>
+      </c>
+      <c r="C14" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="D14" s="9"/>
+      <c r="E14" s="9"/>
+      <c r="F14" s="9"/>
+      <c r="G14" s="9"/>
+      <c r="H14" s="9"/>
+      <c r="I14" s="9"/>
+      <c r="J14" s="9"/>
+      <c r="K14" s="9"/>
+      <c r="L14" s="9"/>
+      <c r="M14" s="9"/>
+      <c r="N14" s="9"/>
+      <c r="O14" s="9"/>
+      <c r="P14" s="10"/>
+      <c r="Q14" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="R14" s="9" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="15" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A15" s="9">
+        <v>16</v>
+      </c>
+      <c r="B15" s="9" t="s">
+        <v>84</v>
+      </c>
+      <c r="C15" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="D15" s="9"/>
+      <c r="E15" s="9"/>
+      <c r="F15" s="9"/>
+      <c r="G15" s="9"/>
+      <c r="H15" s="9"/>
+      <c r="I15" s="9"/>
+      <c r="J15" s="9"/>
+      <c r="K15" s="9"/>
+      <c r="L15" s="9"/>
+      <c r="M15" s="9"/>
+      <c r="N15" s="9"/>
+      <c r="O15" s="9"/>
+      <c r="P15" s="10"/>
+      <c r="Q15" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="R15" s="9" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="16" spans="1:18" ht="18" x14ac:dyDescent="0.25">
+      <c r="A16" s="5">
+        <v>34</v>
+      </c>
+      <c r="B16" s="5" t="s">
+        <v>85</v>
+      </c>
+      <c r="C16" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="D16" s="5"/>
+      <c r="E16" s="5"/>
+      <c r="F16" s="5"/>
+      <c r="G16" s="5"/>
+      <c r="H16" s="5"/>
+      <c r="I16" s="5"/>
+      <c r="J16" s="5"/>
+      <c r="K16" s="5"/>
+      <c r="L16" s="5"/>
+      <c r="M16" s="5"/>
+      <c r="N16" s="5"/>
+      <c r="O16" s="5"/>
+      <c r="P16" s="6"/>
+      <c r="Q16" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="R16" s="5" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="17" spans="1:18" ht="18" x14ac:dyDescent="0.25">
+      <c r="A17" s="5">
+        <v>34</v>
+      </c>
+      <c r="B17" s="5" t="s">
+        <v>85</v>
+      </c>
+      <c r="C17" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="D17" s="5"/>
+      <c r="E17" s="5"/>
+      <c r="F17" s="5"/>
+      <c r="G17" s="5"/>
+      <c r="H17" s="5"/>
+      <c r="I17" s="5"/>
+      <c r="J17" s="5"/>
+      <c r="K17" s="5"/>
+      <c r="L17" s="5"/>
+      <c r="M17" s="5"/>
+      <c r="N17" s="5"/>
+      <c r="O17" s="5"/>
+      <c r="P17" s="6"/>
+      <c r="Q17" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="R17" s="5" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="18" spans="1:18" ht="18" x14ac:dyDescent="0.25">
+      <c r="A18" s="5">
+        <v>34</v>
+      </c>
+      <c r="B18" s="5" t="s">
+        <v>85</v>
+      </c>
+      <c r="C18" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="D18" s="5"/>
+      <c r="E18" s="5"/>
+      <c r="F18" s="5"/>
+      <c r="G18" s="5"/>
+      <c r="H18" s="5"/>
+      <c r="I18" s="5"/>
+      <c r="J18" s="5"/>
+      <c r="K18" s="5"/>
+      <c r="L18" s="5"/>
+      <c r="M18" s="5"/>
+      <c r="N18" s="5"/>
+      <c r="O18" s="5"/>
+      <c r="P18" s="6"/>
+      <c r="Q18" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="R18" s="5" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="19" spans="1:18" ht="18" x14ac:dyDescent="0.25">
+      <c r="A19" s="5">
+        <v>34</v>
+      </c>
+      <c r="B19" s="5" t="s">
+        <v>85</v>
+      </c>
+      <c r="C19" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="D19" s="5"/>
+      <c r="E19" s="5"/>
+      <c r="F19" s="5"/>
+      <c r="G19" s="5"/>
+      <c r="H19" s="5"/>
+      <c r="I19" s="5"/>
+      <c r="J19" s="5"/>
+      <c r="K19" s="5"/>
+      <c r="L19" s="5"/>
+      <c r="M19" s="5"/>
+      <c r="N19" s="5"/>
+      <c r="O19" s="5"/>
+      <c r="P19" s="6"/>
+      <c r="Q19" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="R19" s="5" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="20" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A20" s="9">
+        <v>9</v>
+      </c>
+      <c r="B20" s="9" t="s">
+        <v>86</v>
+      </c>
+      <c r="C20" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="D20" s="9"/>
+      <c r="E20" s="9"/>
+      <c r="F20" s="9"/>
+      <c r="G20" s="9"/>
+      <c r="H20" s="9"/>
+      <c r="I20" s="9"/>
+      <c r="J20" s="9"/>
+      <c r="K20" s="9"/>
+      <c r="L20" s="9"/>
+      <c r="M20" s="9"/>
+      <c r="N20" s="9"/>
+      <c r="O20" s="9"/>
+      <c r="P20" s="10"/>
+      <c r="Q20" s="9" t="s">
+        <v>48</v>
+      </c>
+      <c r="R20" s="9" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="21" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A21" s="9">
+        <v>9</v>
+      </c>
+      <c r="B21" s="9" t="s">
+        <v>86</v>
+      </c>
+      <c r="C21" s="9" t="s">
+        <v>54</v>
+      </c>
+      <c r="D21" s="9"/>
+      <c r="E21" s="9"/>
+      <c r="F21" s="9"/>
+      <c r="G21" s="9"/>
+      <c r="H21" s="9"/>
+      <c r="I21" s="9"/>
+      <c r="J21" s="9"/>
+      <c r="K21" s="9"/>
+      <c r="L21" s="9"/>
+      <c r="M21" s="9"/>
+      <c r="N21" s="9"/>
+      <c r="O21" s="9"/>
+      <c r="P21" s="10"/>
+      <c r="Q21" s="9" t="s">
+        <v>48</v>
+      </c>
+      <c r="R21" s="9" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="22" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A22" s="9">
+        <v>9</v>
+      </c>
+      <c r="B22" s="9" t="s">
+        <v>86</v>
+      </c>
+      <c r="C22" s="9" t="s">
+        <v>47</v>
+      </c>
+      <c r="D22" s="9"/>
+      <c r="E22" s="9"/>
+      <c r="F22" s="9"/>
+      <c r="G22" s="9"/>
+      <c r="H22" s="9"/>
+      <c r="I22" s="9"/>
+      <c r="J22" s="9"/>
+      <c r="K22" s="9"/>
+      <c r="L22" s="9"/>
+      <c r="M22" s="9"/>
+      <c r="N22" s="9"/>
+      <c r="O22" s="9"/>
+      <c r="P22" s="10"/>
+      <c r="Q22" s="9" t="s">
+        <v>48</v>
+      </c>
+      <c r="R22" s="9" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="23" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A23" s="9">
+        <v>9</v>
+      </c>
+      <c r="B23" s="9" t="s">
+        <v>86</v>
+      </c>
+      <c r="C23" s="9" t="s">
+        <v>55</v>
+      </c>
+      <c r="D23" s="9"/>
+      <c r="E23" s="9"/>
+      <c r="F23" s="9"/>
+      <c r="G23" s="9"/>
+      <c r="H23" s="9"/>
+      <c r="I23" s="9"/>
+      <c r="J23" s="9"/>
+      <c r="K23" s="9"/>
+      <c r="L23" s="9"/>
+      <c r="M23" s="9"/>
+      <c r="N23" s="9"/>
+      <c r="O23" s="9"/>
+      <c r="P23" s="10"/>
+      <c r="Q23" s="9" t="s">
+        <v>48</v>
+      </c>
+      <c r="R23" s="9" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="24" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A24" s="9">
+        <v>9</v>
+      </c>
+      <c r="B24" s="9" t="s">
+        <v>86</v>
+      </c>
+      <c r="C24" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="D24" s="9"/>
+      <c r="E24" s="9"/>
+      <c r="F24" s="9"/>
+      <c r="G24" s="9"/>
+      <c r="H24" s="9"/>
+      <c r="I24" s="9"/>
+      <c r="J24" s="9"/>
+      <c r="K24" s="9"/>
+      <c r="L24" s="9"/>
+      <c r="M24" s="9"/>
+      <c r="N24" s="9"/>
+      <c r="O24" s="9"/>
+      <c r="P24" s="10"/>
+      <c r="Q24" s="9" t="s">
+        <v>48</v>
+      </c>
+      <c r="R24" s="9" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="25" spans="1:18" ht="18" x14ac:dyDescent="0.25">
+      <c r="A25" s="9">
+        <v>9</v>
+      </c>
+      <c r="B25" s="9" t="s">
+        <v>86</v>
+      </c>
+      <c r="C25" s="9" t="s">
+        <v>39</v>
+      </c>
+      <c r="D25" s="9"/>
+      <c r="E25" s="9"/>
+      <c r="F25" s="9"/>
+      <c r="G25" s="9"/>
+      <c r="H25" s="9"/>
+      <c r="I25" s="9"/>
+      <c r="J25" s="9"/>
+      <c r="K25" s="9"/>
+      <c r="L25" s="9"/>
+      <c r="M25" s="9"/>
+      <c r="N25" s="9"/>
+      <c r="O25" s="9"/>
+      <c r="P25" s="10"/>
+      <c r="Q25" s="9" t="s">
+        <v>48</v>
+      </c>
+      <c r="R25" s="9" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="26" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A26" s="9">
+        <v>9</v>
+      </c>
+      <c r="B26" s="9" t="s">
+        <v>86</v>
+      </c>
+      <c r="C26" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="D26" s="9"/>
+      <c r="E26" s="9"/>
+      <c r="F26" s="9"/>
+      <c r="G26" s="9"/>
+      <c r="H26" s="9"/>
+      <c r="I26" s="9"/>
+      <c r="J26" s="9"/>
+      <c r="K26" s="9"/>
+      <c r="L26" s="9"/>
+      <c r="M26" s="9"/>
+      <c r="N26" s="9"/>
+      <c r="O26" s="9"/>
+      <c r="P26" s="10"/>
+      <c r="Q26" s="9" t="s">
+        <v>48</v>
+      </c>
+      <c r="R26" s="9" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="27" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A27" s="9">
+        <v>9</v>
+      </c>
+      <c r="B27" s="9" t="s">
+        <v>86</v>
+      </c>
+      <c r="C27" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="D27" s="9"/>
+      <c r="E27" s="9"/>
+      <c r="F27" s="9"/>
+      <c r="G27" s="9"/>
+      <c r="H27" s="9"/>
+      <c r="I27" s="9"/>
+      <c r="J27" s="9"/>
+      <c r="K27" s="9"/>
+      <c r="L27" s="9"/>
+      <c r="M27" s="9"/>
+      <c r="N27" s="9"/>
+      <c r="O27" s="9"/>
+      <c r="P27" s="10"/>
+      <c r="Q27" s="9" t="s">
+        <v>48</v>
+      </c>
+      <c r="R27" s="9" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="28" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A28" s="5">
+        <v>19</v>
+      </c>
+      <c r="B28" s="5" t="s">
+        <v>87</v>
+      </c>
+      <c r="C28" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="D28" s="5"/>
+      <c r="E28" s="5"/>
+      <c r="F28" s="5"/>
+      <c r="G28" s="5"/>
+      <c r="H28" s="5"/>
+      <c r="I28" s="5"/>
+      <c r="J28" s="5"/>
+      <c r="K28" s="5"/>
+      <c r="L28" s="5"/>
+      <c r="M28" s="5"/>
+      <c r="N28" s="5"/>
+      <c r="O28" s="5"/>
+      <c r="P28" s="6"/>
+      <c r="Q28" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="R28" s="5" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="29" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A29" s="5">
+        <v>19</v>
+      </c>
+      <c r="B29" s="5" t="s">
+        <v>87</v>
+      </c>
+      <c r="C29" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="D29" s="5"/>
+      <c r="E29" s="5"/>
+      <c r="F29" s="5"/>
+      <c r="G29" s="5"/>
+      <c r="H29" s="5"/>
+      <c r="I29" s="5"/>
+      <c r="J29" s="5"/>
+      <c r="K29" s="5"/>
+      <c r="L29" s="5"/>
+      <c r="M29" s="5"/>
+      <c r="N29" s="5"/>
+      <c r="O29" s="5"/>
+      <c r="P29" s="6"/>
+      <c r="Q29" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="R29" s="5" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="30" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A30" s="5">
+        <v>19</v>
+      </c>
+      <c r="B30" s="5" t="s">
+        <v>87</v>
+      </c>
+      <c r="C30" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="D30" s="5"/>
+      <c r="E30" s="5"/>
+      <c r="F30" s="5"/>
+      <c r="G30" s="5"/>
+      <c r="H30" s="5"/>
+      <c r="I30" s="5"/>
+      <c r="J30" s="5"/>
+      <c r="K30" s="5"/>
+      <c r="L30" s="5"/>
+      <c r="M30" s="5"/>
+      <c r="N30" s="5"/>
+      <c r="O30" s="5"/>
+      <c r="P30" s="6"/>
+      <c r="Q30" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="R30" s="5" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="31" spans="1:18" ht="18" x14ac:dyDescent="0.25">
+      <c r="A31" s="5">
+        <v>19</v>
+      </c>
+      <c r="B31" s="5" t="s">
+        <v>87</v>
+      </c>
+      <c r="C31" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="D31" s="5"/>
+      <c r="E31" s="5"/>
+      <c r="F31" s="5"/>
+      <c r="G31" s="5"/>
+      <c r="H31" s="5"/>
+      <c r="I31" s="5"/>
+      <c r="J31" s="5"/>
+      <c r="K31" s="5"/>
+      <c r="L31" s="5"/>
+      <c r="M31" s="5"/>
+      <c r="N31" s="5"/>
+      <c r="O31" s="5"/>
+      <c r="P31" s="6"/>
+      <c r="Q31" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="R31" s="5" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="32" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A32" s="5">
+        <v>19</v>
+      </c>
+      <c r="B32" s="5" t="s">
+        <v>87</v>
+      </c>
+      <c r="C32" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="D32" s="5"/>
+      <c r="E32" s="5"/>
+      <c r="F32" s="5"/>
+      <c r="G32" s="5"/>
+      <c r="H32" s="5"/>
+      <c r="I32" s="5"/>
+      <c r="J32" s="5"/>
+      <c r="K32" s="5"/>
+      <c r="L32" s="5"/>
+      <c r="M32" s="5"/>
+      <c r="N32" s="5"/>
+      <c r="O32" s="5"/>
+      <c r="P32" s="6"/>
+      <c r="Q32" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="R32" s="5" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="33" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A33" s="5">
+        <v>19</v>
+      </c>
+      <c r="B33" s="5" t="s">
+        <v>87</v>
+      </c>
+      <c r="C33" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="D33" s="5"/>
+      <c r="E33" s="5"/>
+      <c r="F33" s="5"/>
+      <c r="G33" s="5"/>
+      <c r="H33" s="5"/>
+      <c r="I33" s="5"/>
+      <c r="J33" s="5"/>
+      <c r="K33" s="5"/>
+      <c r="L33" s="5"/>
+      <c r="M33" s="5"/>
+      <c r="N33" s="5"/>
+      <c r="O33" s="5"/>
+      <c r="P33" s="6"/>
+      <c r="Q33" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="R33" s="5" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="34" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A34" s="5">
+        <v>19</v>
+      </c>
+      <c r="B34" s="5" t="s">
+        <v>87</v>
+      </c>
+      <c r="C34" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="D34" s="5"/>
+      <c r="E34" s="5"/>
+      <c r="F34" s="5"/>
+      <c r="G34" s="5"/>
+      <c r="H34" s="5"/>
+      <c r="I34" s="5"/>
+      <c r="J34" s="5"/>
+      <c r="K34" s="5"/>
+      <c r="L34" s="5"/>
+      <c r="M34" s="5"/>
+      <c r="N34" s="5"/>
+      <c r="O34" s="5"/>
+      <c r="P34" s="6"/>
+      <c r="Q34" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="R34" s="5" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="35" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A35" s="5">
+        <v>19</v>
+      </c>
+      <c r="B35" s="5" t="s">
+        <v>87</v>
+      </c>
+      <c r="C35" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="D35" s="5"/>
+      <c r="E35" s="5"/>
+      <c r="F35" s="5"/>
+      <c r="G35" s="5"/>
+      <c r="H35" s="5"/>
+      <c r="I35" s="5"/>
+      <c r="J35" s="5"/>
+      <c r="K35" s="5"/>
+      <c r="L35" s="5"/>
+      <c r="M35" s="5"/>
+      <c r="N35" s="5"/>
+      <c r="O35" s="5"/>
+      <c r="P35" s="6"/>
+      <c r="Q35" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="R35" s="5" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="36" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A36" s="5">
+        <v>19</v>
+      </c>
+      <c r="B36" s="5" t="s">
+        <v>87</v>
+      </c>
+      <c r="C36" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="D36" s="5"/>
+      <c r="E36" s="5"/>
+      <c r="F36" s="5"/>
+      <c r="G36" s="5"/>
+      <c r="H36" s="5"/>
+      <c r="I36" s="5"/>
+      <c r="J36" s="5"/>
+      <c r="K36" s="5"/>
+      <c r="L36" s="5"/>
+      <c r="M36" s="5"/>
+      <c r="N36" s="5"/>
+      <c r="O36" s="5"/>
+      <c r="P36" s="6"/>
+      <c r="Q36" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="R36" s="5" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="37" spans="1:18" ht="18" x14ac:dyDescent="0.25">
+      <c r="A37" s="5">
+        <v>19</v>
+      </c>
+      <c r="B37" s="5" t="s">
+        <v>87</v>
+      </c>
+      <c r="C37" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="D37" s="5"/>
+      <c r="E37" s="5"/>
+      <c r="F37" s="5"/>
+      <c r="G37" s="5"/>
+      <c r="H37" s="5"/>
+      <c r="I37" s="5"/>
+      <c r="J37" s="5"/>
+      <c r="K37" s="5"/>
+      <c r="L37" s="5"/>
+      <c r="M37" s="5"/>
+      <c r="N37" s="5"/>
+      <c r="O37" s="5"/>
+      <c r="P37" s="6"/>
+      <c r="Q37" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="R37" s="5" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="38" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A38" s="9">
+        <v>17</v>
+      </c>
+      <c r="B38" s="9" t="s">
+        <v>89</v>
+      </c>
+      <c r="C38" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="D38" s="9"/>
+      <c r="E38" s="9"/>
+      <c r="F38" s="9"/>
+      <c r="G38" s="9"/>
+      <c r="H38" s="9"/>
+      <c r="I38" s="9"/>
+      <c r="J38" s="9"/>
+      <c r="K38" s="9"/>
+      <c r="L38" s="9"/>
+      <c r="M38" s="9"/>
+      <c r="N38" s="9"/>
+      <c r="O38" s="9"/>
+      <c r="P38" s="10"/>
+      <c r="Q38" s="9" t="s">
+        <v>38</v>
+      </c>
+      <c r="R38" s="9" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="39" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A39" s="9">
+        <v>17</v>
+      </c>
+      <c r="B39" s="9" t="s">
+        <v>89</v>
+      </c>
+      <c r="C39" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="D39" s="9"/>
+      <c r="E39" s="9"/>
+      <c r="F39" s="9"/>
+      <c r="G39" s="9"/>
+      <c r="H39" s="9"/>
+      <c r="I39" s="9"/>
+      <c r="J39" s="9"/>
+      <c r="K39" s="9"/>
+      <c r="L39" s="9"/>
+      <c r="M39" s="9"/>
+      <c r="N39" s="9"/>
+      <c r="O39" s="9"/>
+      <c r="P39" s="10"/>
+      <c r="Q39" s="9" t="s">
+        <v>38</v>
+      </c>
+      <c r="R39" s="9" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="40" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A40" s="9">
+        <v>17</v>
+      </c>
+      <c r="B40" s="9" t="s">
+        <v>89</v>
+      </c>
+      <c r="C40" s="9" t="s">
+        <v>22</v>
+      </c>
+      <c r="D40" s="9"/>
+      <c r="E40" s="9"/>
+      <c r="F40" s="9"/>
+      <c r="G40" s="9"/>
+      <c r="H40" s="9"/>
+      <c r="I40" s="9"/>
+      <c r="J40" s="9"/>
+      <c r="K40" s="9"/>
+      <c r="L40" s="9"/>
+      <c r="M40" s="9"/>
+      <c r="N40" s="9"/>
+      <c r="O40" s="9"/>
+      <c r="P40" s="10"/>
+      <c r="Q40" s="9" t="s">
+        <v>38</v>
+      </c>
+      <c r="R40" s="9" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="41" spans="1:18" ht="18" x14ac:dyDescent="0.25">
+      <c r="A41" s="9">
+        <v>17</v>
+      </c>
+      <c r="B41" s="9" t="s">
+        <v>89</v>
+      </c>
+      <c r="C41" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="D41" s="9"/>
+      <c r="E41" s="9"/>
+      <c r="F41" s="9"/>
+      <c r="G41" s="9"/>
+      <c r="H41" s="9"/>
+      <c r="I41" s="9"/>
+      <c r="J41" s="9"/>
+      <c r="K41" s="9"/>
+      <c r="L41" s="9"/>
+      <c r="M41" s="9"/>
+      <c r="N41" s="9"/>
+      <c r="O41" s="9"/>
+      <c r="P41" s="10"/>
+      <c r="Q41" s="9" t="s">
+        <v>38</v>
+      </c>
+      <c r="R41" s="9" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="42" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A42" s="9">
+        <v>17</v>
+      </c>
+      <c r="B42" s="9" t="s">
+        <v>89</v>
+      </c>
+      <c r="C42" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="D42" s="9"/>
+      <c r="E42" s="9"/>
+      <c r="F42" s="9"/>
+      <c r="G42" s="9"/>
+      <c r="H42" s="9"/>
+      <c r="I42" s="9"/>
+      <c r="J42" s="9"/>
+      <c r="K42" s="9"/>
+      <c r="L42" s="9"/>
+      <c r="M42" s="9"/>
+      <c r="N42" s="9"/>
+      <c r="O42" s="9"/>
+      <c r="P42" s="10"/>
+      <c r="Q42" s="9" t="s">
+        <v>38</v>
+      </c>
+      <c r="R42" s="9" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="43" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A43" s="9">
+        <v>17</v>
+      </c>
+      <c r="B43" s="9" t="s">
+        <v>89</v>
+      </c>
+      <c r="C43" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="D43" s="9"/>
+      <c r="E43" s="9"/>
+      <c r="F43" s="9"/>
+      <c r="G43" s="9"/>
+      <c r="H43" s="9"/>
+      <c r="I43" s="9"/>
+      <c r="J43" s="9"/>
+      <c r="K43" s="9"/>
+      <c r="L43" s="9"/>
+      <c r="M43" s="9"/>
+      <c r="N43" s="9"/>
+      <c r="O43" s="9"/>
+      <c r="P43" s="10"/>
+      <c r="Q43" s="9" t="s">
+        <v>38</v>
+      </c>
+      <c r="R43" s="9" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="44" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A44" s="9">
+        <v>17</v>
+      </c>
+      <c r="B44" s="9" t="s">
+        <v>89</v>
+      </c>
+      <c r="C44" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="D44" s="9"/>
+      <c r="E44" s="9"/>
+      <c r="F44" s="9"/>
+      <c r="G44" s="9"/>
+      <c r="H44" s="9"/>
+      <c r="I44" s="9"/>
+      <c r="J44" s="9"/>
+      <c r="K44" s="9"/>
+      <c r="L44" s="9"/>
+      <c r="M44" s="9"/>
+      <c r="N44" s="9"/>
+      <c r="O44" s="9"/>
+      <c r="P44" s="10"/>
+      <c r="Q44" s="9" t="s">
+        <v>38</v>
+      </c>
+      <c r="R44" s="9" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="45" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A45" s="9">
+        <v>17</v>
+      </c>
+      <c r="B45" s="9" t="s">
+        <v>89</v>
+      </c>
+      <c r="C45" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="D45" s="9"/>
+      <c r="E45" s="9"/>
+      <c r="F45" s="9"/>
+      <c r="G45" s="9"/>
+      <c r="H45" s="9"/>
+      <c r="I45" s="9"/>
+      <c r="J45" s="9"/>
+      <c r="K45" s="9"/>
+      <c r="L45" s="9"/>
+      <c r="M45" s="9"/>
+      <c r="N45" s="9"/>
+      <c r="O45" s="9"/>
+      <c r="P45" s="10"/>
+      <c r="Q45" s="9" t="s">
+        <v>38</v>
+      </c>
+      <c r="R45" s="9" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="46" spans="1:18" ht="18" x14ac:dyDescent="0.25">
+      <c r="A46" s="9">
+        <v>17</v>
+      </c>
+      <c r="B46" s="9" t="s">
+        <v>89</v>
+      </c>
+      <c r="C46" s="9" t="s">
+        <v>39</v>
+      </c>
+      <c r="D46" s="9"/>
+      <c r="E46" s="9"/>
+      <c r="F46" s="9"/>
+      <c r="G46" s="9"/>
+      <c r="H46" s="9"/>
+      <c r="I46" s="9"/>
+      <c r="J46" s="9"/>
+      <c r="K46" s="9"/>
+      <c r="L46" s="9"/>
+      <c r="M46" s="9"/>
+      <c r="N46" s="9"/>
+      <c r="O46" s="9"/>
+      <c r="P46" s="10"/>
+      <c r="Q46" s="9" t="s">
+        <v>38</v>
+      </c>
+      <c r="R46" s="9" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="47" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A47" s="9">
+        <v>17</v>
+      </c>
+      <c r="B47" s="9" t="s">
+        <v>89</v>
+      </c>
+      <c r="C47" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="D47" s="9"/>
+      <c r="E47" s="9"/>
+      <c r="F47" s="9"/>
+      <c r="G47" s="9"/>
+      <c r="H47" s="9"/>
+      <c r="I47" s="9"/>
+      <c r="J47" s="9"/>
+      <c r="K47" s="9"/>
+      <c r="L47" s="9"/>
+      <c r="M47" s="9"/>
+      <c r="N47" s="9"/>
+      <c r="O47" s="9"/>
+      <c r="P47" s="10"/>
+      <c r="Q47" s="9" t="s">
+        <v>38</v>
+      </c>
+      <c r="R47" s="9" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="48" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A48" s="5">
+        <v>30</v>
+      </c>
+      <c r="B48" s="5" t="s">
+        <v>90</v>
+      </c>
+      <c r="C48" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="D48" s="5"/>
+      <c r="E48" s="5"/>
+      <c r="F48" s="5"/>
+      <c r="G48" s="5"/>
+      <c r="H48" s="5"/>
+      <c r="I48" s="5"/>
+      <c r="J48" s="5"/>
+      <c r="K48" s="5"/>
+      <c r="L48" s="5"/>
+      <c r="M48" s="5"/>
+      <c r="N48" s="5"/>
+      <c r="O48" s="5"/>
+      <c r="P48" s="6"/>
+      <c r="Q48" s="5" t="s">
+        <v>70</v>
+      </c>
+      <c r="R48" s="5" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="49" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A49" s="5">
+        <v>30</v>
+      </c>
+      <c r="B49" s="5" t="s">
+        <v>90</v>
+      </c>
+      <c r="C49" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="D49" s="7"/>
+      <c r="E49" s="7"/>
+      <c r="F49" s="7"/>
+      <c r="G49" s="7"/>
+      <c r="H49" s="7"/>
+      <c r="I49" s="7"/>
+      <c r="J49" s="7"/>
+      <c r="K49" s="7"/>
+      <c r="L49" s="7"/>
+      <c r="M49" s="7"/>
+      <c r="N49" s="7"/>
+      <c r="O49" s="7"/>
+      <c r="P49" s="6"/>
+      <c r="Q49" s="5" t="s">
+        <v>70</v>
+      </c>
+      <c r="R49" s="5" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="50" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A50" s="5">
+        <v>30</v>
+      </c>
+      <c r="B50" s="5" t="s">
+        <v>90</v>
+      </c>
+      <c r="C50" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="D50" s="5"/>
+      <c r="E50" s="5"/>
+      <c r="F50" s="5"/>
+      <c r="G50" s="5"/>
+      <c r="H50" s="5"/>
+      <c r="I50" s="5"/>
+      <c r="J50" s="5"/>
+      <c r="K50" s="5"/>
+      <c r="L50" s="5"/>
+      <c r="M50" s="5"/>
+      <c r="N50" s="5"/>
+      <c r="O50" s="5"/>
+      <c r="P50" s="6"/>
+      <c r="Q50" s="5" t="s">
+        <v>70</v>
+      </c>
+      <c r="R50" s="5" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="51" spans="1:18" ht="18" x14ac:dyDescent="0.25">
+      <c r="A51" s="5">
+        <v>30</v>
+      </c>
+      <c r="B51" s="5" t="s">
+        <v>90</v>
+      </c>
+      <c r="C51" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="D51" s="5"/>
+      <c r="E51" s="5"/>
+      <c r="F51" s="5"/>
+      <c r="G51" s="5"/>
+      <c r="H51" s="5"/>
+      <c r="I51" s="5"/>
+      <c r="J51" s="5"/>
+      <c r="K51" s="5"/>
+      <c r="L51" s="5"/>
+      <c r="M51" s="5"/>
+      <c r="N51" s="5"/>
+      <c r="O51" s="5"/>
+      <c r="P51" s="6"/>
+      <c r="Q51" s="5" t="s">
+        <v>70</v>
+      </c>
+      <c r="R51" s="5" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="52" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A52" s="5">
+        <v>30</v>
+      </c>
+      <c r="B52" s="5" t="s">
+        <v>90</v>
+      </c>
+      <c r="C52" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="D52" s="5"/>
+      <c r="E52" s="5"/>
+      <c r="F52" s="5"/>
+      <c r="G52" s="5"/>
+      <c r="H52" s="5"/>
+      <c r="I52" s="5"/>
+      <c r="J52" s="5"/>
+      <c r="K52" s="5"/>
+      <c r="L52" s="5"/>
+      <c r="M52" s="5"/>
+      <c r="N52" s="5"/>
+      <c r="O52" s="5"/>
+      <c r="P52" s="6"/>
+      <c r="Q52" s="5" t="s">
+        <v>70</v>
+      </c>
+      <c r="R52" s="5" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="53" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A53" s="5">
+        <v>30</v>
+      </c>
+      <c r="B53" s="5" t="s">
+        <v>90</v>
+      </c>
+      <c r="C53" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="D53" s="7"/>
+      <c r="E53" s="7"/>
+      <c r="F53" s="7"/>
+      <c r="G53" s="7"/>
+      <c r="H53" s="7"/>
+      <c r="I53" s="7"/>
+      <c r="J53" s="7"/>
+      <c r="K53" s="7"/>
+      <c r="L53" s="7"/>
+      <c r="M53" s="7"/>
+      <c r="N53" s="7"/>
+      <c r="O53" s="7"/>
+      <c r="P53" s="6"/>
+      <c r="Q53" s="5" t="s">
+        <v>70</v>
+      </c>
+      <c r="R53" s="5" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="54" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A54" s="5">
+        <v>30</v>
+      </c>
+      <c r="B54" s="5" t="s">
+        <v>90</v>
+      </c>
+      <c r="C54" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="D54" s="5"/>
+      <c r="E54" s="5"/>
+      <c r="F54" s="5"/>
+      <c r="G54" s="5"/>
+      <c r="H54" s="5"/>
+      <c r="I54" s="5"/>
+      <c r="J54" s="5"/>
+      <c r="K54" s="5"/>
+      <c r="L54" s="5"/>
+      <c r="M54" s="5"/>
+      <c r="N54" s="5"/>
+      <c r="O54" s="5"/>
+      <c r="P54" s="6"/>
+      <c r="Q54" s="5" t="s">
+        <v>70</v>
+      </c>
+      <c r="R54" s="5" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="55" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A55" s="5">
+        <v>30</v>
+      </c>
+      <c r="B55" s="5" t="s">
+        <v>90</v>
+      </c>
+      <c r="C55" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="D55" s="5"/>
+      <c r="E55" s="5"/>
+      <c r="F55" s="5"/>
+      <c r="G55" s="5"/>
+      <c r="H55" s="5"/>
+      <c r="I55" s="5"/>
+      <c r="J55" s="5"/>
+      <c r="K55" s="5"/>
+      <c r="L55" s="5"/>
+      <c r="M55" s="5"/>
+      <c r="N55" s="5"/>
+      <c r="O55" s="5"/>
+      <c r="P55" s="6"/>
+      <c r="Q55" s="5" t="s">
+        <v>70</v>
+      </c>
+      <c r="R55" s="5" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="56" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A56" s="5">
+        <v>30</v>
+      </c>
+      <c r="B56" s="5" t="s">
+        <v>90</v>
+      </c>
+      <c r="C56" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="D56" s="5"/>
+      <c r="E56" s="5"/>
+      <c r="F56" s="5"/>
+      <c r="G56" s="5"/>
+      <c r="H56" s="5"/>
+      <c r="I56" s="5"/>
+      <c r="J56" s="5"/>
+      <c r="K56" s="5"/>
+      <c r="L56" s="5"/>
+      <c r="M56" s="5"/>
+      <c r="N56" s="5"/>
+      <c r="O56" s="5"/>
+      <c r="P56" s="6"/>
+      <c r="Q56" s="5" t="s">
+        <v>70</v>
+      </c>
+      <c r="R56" s="5" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="57" spans="1:18" ht="18" x14ac:dyDescent="0.25">
+      <c r="A57" s="5">
+        <v>30</v>
+      </c>
+      <c r="B57" s="5" t="s">
+        <v>90</v>
+      </c>
+      <c r="C57" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="D57" s="5"/>
+      <c r="E57" s="5"/>
+      <c r="F57" s="5"/>
+      <c r="G57" s="5"/>
+      <c r="H57" s="5"/>
+      <c r="I57" s="5"/>
+      <c r="J57" s="5"/>
+      <c r="K57" s="5"/>
+      <c r="L57" s="5"/>
+      <c r="M57" s="5"/>
+      <c r="N57" s="5"/>
+      <c r="O57" s="5"/>
+      <c r="P57" s="6"/>
+      <c r="Q57" s="5" t="s">
+        <v>70</v>
+      </c>
+      <c r="R57" s="5" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="58" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A58" s="9">
+        <v>11</v>
+      </c>
+      <c r="B58" s="9" t="s">
+        <v>91</v>
+      </c>
+      <c r="C58" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="D58" s="9"/>
+      <c r="E58" s="9"/>
+      <c r="F58" s="9"/>
+      <c r="G58" s="9"/>
+      <c r="H58" s="9"/>
+      <c r="I58" s="9"/>
+      <c r="J58" s="9"/>
+      <c r="K58" s="9"/>
+      <c r="L58" s="9"/>
+      <c r="M58" s="9"/>
+      <c r="N58" s="9"/>
+      <c r="O58" s="9"/>
+      <c r="P58" s="10"/>
+      <c r="Q58" s="9" t="s">
+        <v>77</v>
+      </c>
+      <c r="R58" s="9" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="59" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A59" s="9">
+        <v>11</v>
+      </c>
+      <c r="B59" s="9" t="s">
+        <v>91</v>
+      </c>
+      <c r="C59" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="D59" s="9"/>
+      <c r="E59" s="9"/>
+      <c r="F59" s="9"/>
+      <c r="G59" s="9"/>
+      <c r="H59" s="9"/>
+      <c r="I59" s="9"/>
+      <c r="J59" s="9"/>
+      <c r="K59" s="9"/>
+      <c r="L59" s="9"/>
+      <c r="M59" s="9"/>
+      <c r="N59" s="9"/>
+      <c r="O59" s="9"/>
+      <c r="P59" s="10"/>
+      <c r="Q59" s="9" t="s">
+        <v>77</v>
+      </c>
+      <c r="R59" s="9" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="60" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A60" s="9">
+        <v>11</v>
+      </c>
+      <c r="B60" s="9" t="s">
+        <v>91</v>
+      </c>
+      <c r="C60" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="D60" s="9"/>
+      <c r="E60" s="9"/>
+      <c r="F60" s="9"/>
+      <c r="G60" s="9"/>
+      <c r="H60" s="9"/>
+      <c r="I60" s="9"/>
+      <c r="J60" s="9"/>
+      <c r="K60" s="9"/>
+      <c r="L60" s="9"/>
+      <c r="M60" s="9"/>
+      <c r="N60" s="9"/>
+      <c r="O60" s="9"/>
+      <c r="P60" s="10"/>
+      <c r="Q60" s="9" t="s">
+        <v>77</v>
+      </c>
+      <c r="R60" s="9" t="s">
+        <v>82</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+</worksheet>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="f76aa77c-8923-4724-9a6d-d588cc513697">
@@ -19663,6 +21502,15 @@
     <TaxCatchAll xmlns="89c54d5b-05ac-45d5-9242-aabb385cc5ad" xsi:nil="true"/>
   </documentManagement>
 </p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -19861,14 +21709,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F5CFE981-CBAC-4360-B0CE-AB3235A33930}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F919D1BA-3E11-4877-AEE4-5A5340B7B50A}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
@@ -19881,6 +21721,14 @@
     <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
     <ds:schemaRef ds:uri="f76aa77c-8923-4724-9a6d-d588cc513697"/>
     <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F5CFE981-CBAC-4360-B0CE-AB3235A33930}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>

<commit_message>
Base CNH atualizada — 24/08/2026 12:07
</commit_message>
<xml_diff>
--- a/dados/metas.xlsx
+++ b/dados/metas.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pedro.sa\Documents\dashboard-oportunidades\dados\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B9A8B9C1-ECF7-45B3-ADB9-1CA88A09E1B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B755A52D-C568-49CC-A673-48E3C2CBDC18}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1482" uniqueCount="93">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1498" uniqueCount="94">
   <si>
     <t>CÓD</t>
   </si>
@@ -320,6 +320,9 @@
   </si>
   <si>
     <t>WESLEY.LIMA</t>
+  </si>
+  <si>
+    <t>HUGO.MOL</t>
   </si>
 </sst>
 </file>
@@ -731,7 +734,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:R240"/>
+  <dimension ref="A1:R244"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.140625" style="4"/>
@@ -849,7 +852,7 @@
         <v>32</v>
       </c>
       <c r="R2" s="4" t="s">
-        <v>21</v>
+        <v>34</v>
       </c>
     </row>
     <row r="3" spans="1:18" x14ac:dyDescent="0.25">
@@ -905,7 +908,7 @@
         <v>32</v>
       </c>
       <c r="R3" s="4" t="s">
-        <v>21</v>
+        <v>34</v>
       </c>
     </row>
     <row r="4" spans="1:18" x14ac:dyDescent="0.25">
@@ -961,7 +964,7 @@
         <v>32</v>
       </c>
       <c r="R4" s="4" t="s">
-        <v>21</v>
+        <v>34</v>
       </c>
     </row>
     <row r="5" spans="1:18" x14ac:dyDescent="0.25">
@@ -1017,7 +1020,7 @@
         <v>32</v>
       </c>
       <c r="R5" s="4" t="s">
-        <v>21</v>
+        <v>34</v>
       </c>
     </row>
     <row r="6" spans="1:18" x14ac:dyDescent="0.25">
@@ -4545,7 +4548,7 @@
         <v>20</v>
       </c>
       <c r="R68" s="4" t="s">
-        <v>21</v>
+        <v>34</v>
       </c>
     </row>
     <row r="69" spans="1:18" x14ac:dyDescent="0.25">
@@ -4601,7 +4604,7 @@
         <v>20</v>
       </c>
       <c r="R69" s="4" t="s">
-        <v>21</v>
+        <v>34</v>
       </c>
     </row>
     <row r="70" spans="1:18" x14ac:dyDescent="0.25">
@@ -4657,7 +4660,7 @@
         <v>20</v>
       </c>
       <c r="R70" s="4" t="s">
-        <v>21</v>
+        <v>34</v>
       </c>
     </row>
     <row r="71" spans="1:18" x14ac:dyDescent="0.25">
@@ -4713,7 +4716,7 @@
         <v>20</v>
       </c>
       <c r="R71" s="4" t="s">
-        <v>21</v>
+        <v>34</v>
       </c>
     </row>
     <row r="72" spans="1:18" x14ac:dyDescent="0.25">
@@ -4769,7 +4772,7 @@
         <v>20</v>
       </c>
       <c r="R72" s="4" t="s">
-        <v>21</v>
+        <v>34</v>
       </c>
     </row>
     <row r="73" spans="1:18" x14ac:dyDescent="0.25">
@@ -4825,7 +4828,7 @@
         <v>20</v>
       </c>
       <c r="R73" s="4" t="s">
-        <v>21</v>
+        <v>34</v>
       </c>
     </row>
     <row r="74" spans="1:18" x14ac:dyDescent="0.25">
@@ -4881,7 +4884,7 @@
         <v>20</v>
       </c>
       <c r="R74" s="4" t="s">
-        <v>21</v>
+        <v>34</v>
       </c>
     </row>
     <row r="75" spans="1:18" x14ac:dyDescent="0.25">
@@ -4937,7 +4940,7 @@
         <v>20</v>
       </c>
       <c r="R75" s="4" t="s">
-        <v>21</v>
+        <v>34</v>
       </c>
     </row>
     <row r="76" spans="1:18" x14ac:dyDescent="0.25">
@@ -4993,7 +4996,7 @@
         <v>20</v>
       </c>
       <c r="R76" s="4" t="s">
-        <v>21</v>
+        <v>34</v>
       </c>
     </row>
     <row r="77" spans="1:18" x14ac:dyDescent="0.25">
@@ -14030,12 +14033,148 @@
         <v>21</v>
       </c>
     </row>
+    <row r="241" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A241" s="4">
+        <v>40011</v>
+      </c>
+      <c r="B241" s="4" t="s">
+        <v>93</v>
+      </c>
+      <c r="C241" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="K241" s="4">
+        <v>0</v>
+      </c>
+      <c r="L241" s="4">
+        <v>0</v>
+      </c>
+      <c r="M241" s="4">
+        <v>1</v>
+      </c>
+      <c r="N241" s="4">
+        <v>0</v>
+      </c>
+      <c r="O241" s="4">
+        <v>1</v>
+      </c>
+      <c r="P241" s="4">
+        <v>2</v>
+      </c>
+      <c r="Q241" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="R241" s="4" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="242" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A242" s="4">
+        <v>40011</v>
+      </c>
+      <c r="B242" s="4" t="s">
+        <v>93</v>
+      </c>
+      <c r="C242" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="K242" s="4">
+        <v>1</v>
+      </c>
+      <c r="L242" s="4">
+        <v>0</v>
+      </c>
+      <c r="M242" s="4">
+        <v>1</v>
+      </c>
+      <c r="N242" s="4">
+        <v>0</v>
+      </c>
+      <c r="O242" s="4">
+        <v>1</v>
+      </c>
+      <c r="P242" s="4">
+        <v>3</v>
+      </c>
+      <c r="Q242" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="R242" s="4" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="243" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A243" s="4">
+        <v>40011</v>
+      </c>
+      <c r="B243" s="4" t="s">
+        <v>93</v>
+      </c>
+      <c r="C243" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="K243" s="4">
+        <v>100000</v>
+      </c>
+      <c r="L243" s="4">
+        <v>150000</v>
+      </c>
+      <c r="M243" s="4">
+        <v>140000</v>
+      </c>
+      <c r="N243" s="4">
+        <v>120000</v>
+      </c>
+      <c r="O243" s="4">
+        <v>80000</v>
+      </c>
+      <c r="P243" s="4">
+        <v>590000</v>
+      </c>
+      <c r="Q243" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="R243" s="4" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="244" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A244" s="4">
+        <v>40011</v>
+      </c>
+      <c r="B244" s="4" t="s">
+        <v>93</v>
+      </c>
+      <c r="C244" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="K244" s="4">
+        <v>1</v>
+      </c>
+      <c r="L244" s="4">
+        <v>2</v>
+      </c>
+      <c r="M244" s="4">
+        <v>1</v>
+      </c>
+      <c r="N244" s="4">
+        <v>1</v>
+      </c>
+      <c r="O244" s="4">
+        <v>1</v>
+      </c>
+      <c r="P244" s="4">
+        <v>6</v>
+      </c>
+      <c r="Q244" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="R244" s="4" t="s">
+        <v>21</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:R240" xr:uid="{00000000-0001-0000-0000-000000000000}">
-    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:R240">
-      <sortCondition ref="B1:B240"/>
-    </sortState>
-  </autoFilter>
+  <autoFilter ref="A1:R240" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -21576,26 +21715,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="f76aa77c-8923-4724-9a6d-d588cc513697">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="89c54d5b-05ac-45d5-9242-aabb385cc5ad" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100B96036E30F13644F923D207E371C305D" ma:contentTypeVersion="11" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="1d197ceb99055fd1a93a3a14aec1bdd8">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="f76aa77c-8923-4724-9a6d-d588cc513697" xmlns:ns3="89c54d5b-05ac-45d5-9242-aabb385cc5ad" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="5b86266bfd619f312673123d0bd20d23" ns2:_="" ns3:_="">
     <xsd:import namespace="f76aa77c-8923-4724-9a6d-d588cc513697"/>
@@ -21790,32 +21909,27 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F919D1BA-3E11-4877-AEE4-5A5340B7B50A}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="89c54d5b-05ac-45d5-9242-aabb385cc5ad"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="f76aa77c-8923-4724-9a6d-d588cc513697"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F5CFE981-CBAC-4360-B0CE-AB3235A33930}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="f76aa77c-8923-4724-9a6d-d588cc513697">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="89c54d5b-05ac-45d5-9242-aabb385cc5ad" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8BDC8EFC-C946-4B3C-B84E-1270F018751C}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -21832,4 +21946,29 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F5CFE981-CBAC-4360-B0CE-AB3235A33930}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F919D1BA-3E11-4877-AEE4-5A5340B7B50A}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="89c54d5b-05ac-45d5-9242-aabb385cc5ad"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="f76aa77c-8923-4724-9a6d-d588cc513697"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Atualização de base (+ vendas + CNH) — 26/08/2026 11:11
</commit_message>
<xml_diff>
--- a/dados/metas.xlsx
+++ b/dados/metas.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pedro.sa\Documents\dashboard-oportunidades\dados\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D8CE5EEB-0940-4C12-95B5-6FAEAE4AACCE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B5BBD786-9CBC-4E49-8D77-5E5D27E6DDE1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -5003,6 +5003,9 @@
       </c>
     </row>
     <row r="77" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A77" s="4">
+        <v>260044</v>
+      </c>
       <c r="B77" s="4" t="s">
         <v>94</v>
       </c>
@@ -5032,6 +5035,9 @@
       </c>
     </row>
     <row r="78" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A78" s="4">
+        <v>260044</v>
+      </c>
       <c r="B78" s="4" t="s">
         <v>94</v>
       </c>
@@ -5061,6 +5067,9 @@
       </c>
     </row>
     <row r="79" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A79" s="4">
+        <v>260044</v>
+      </c>
       <c r="B79" s="4" t="s">
         <v>94</v>
       </c>
@@ -5090,6 +5099,9 @@
       </c>
     </row>
     <row r="80" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A80" s="4">
+        <v>260044</v>
+      </c>
       <c r="B80" s="4" t="s">
         <v>94</v>
       </c>
@@ -5119,6 +5131,9 @@
       </c>
     </row>
     <row r="81" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A81" s="4">
+        <v>260044</v>
+      </c>
       <c r="B81" s="4" t="s">
         <v>94</v>
       </c>
@@ -5148,6 +5163,9 @@
       </c>
     </row>
     <row r="82" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A82" s="4">
+        <v>260044</v>
+      </c>
       <c r="B82" s="4" t="s">
         <v>94</v>
       </c>
@@ -5177,6 +5195,9 @@
       </c>
     </row>
     <row r="83" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A83" s="4">
+        <v>260044</v>
+      </c>
       <c r="B83" s="4" t="s">
         <v>94</v>
       </c>
@@ -5206,6 +5227,9 @@
       </c>
     </row>
     <row r="84" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A84" s="4">
+        <v>260044</v>
+      </c>
       <c r="B84" s="4" t="s">
         <v>94</v>
       </c>
@@ -5235,6 +5259,9 @@
       </c>
     </row>
     <row r="85" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A85" s="4">
+        <v>260044</v>
+      </c>
       <c r="B85" s="4" t="s">
         <v>94</v>
       </c>

</xml_diff>

<commit_message>
Atualização de base — 31/08/2026 11:14
</commit_message>
<xml_diff>
--- a/dados/metas.xlsx
+++ b/dados/metas.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pedro.sa\Documents\dashboard-oportunidades\dados\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B5BBD786-9CBC-4E49-8D77-5E5D27E6DDE1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{55F1C0CF-59CA-4E66-A1C7-1C85BAE78261}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -11275,7 +11275,7 @@
         <v>38</v>
       </c>
       <c r="R193" s="4" t="s">
-        <v>21</v>
+        <v>34</v>
       </c>
     </row>
     <row r="194" spans="1:18" x14ac:dyDescent="0.25">
@@ -22006,26 +22006,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="f76aa77c-8923-4724-9a6d-d588cc513697">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="89c54d5b-05ac-45d5-9242-aabb385cc5ad" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100B96036E30F13644F923D207E371C305D" ma:contentTypeVersion="11" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="1d197ceb99055fd1a93a3a14aec1bdd8">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="f76aa77c-8923-4724-9a6d-d588cc513697" xmlns:ns3="89c54d5b-05ac-45d5-9242-aabb385cc5ad" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="5b86266bfd619f312673123d0bd20d23" ns2:_="" ns3:_="">
     <xsd:import namespace="f76aa77c-8923-4724-9a6d-d588cc513697"/>
@@ -22220,32 +22200,27 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F919D1BA-3E11-4877-AEE4-5A5340B7B50A}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="89c54d5b-05ac-45d5-9242-aabb385cc5ad"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="f76aa77c-8923-4724-9a6d-d588cc513697"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F5CFE981-CBAC-4360-B0CE-AB3235A33930}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="f76aa77c-8923-4724-9a6d-d588cc513697">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="89c54d5b-05ac-45d5-9242-aabb385cc5ad" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8BDC8EFC-C946-4B3C-B84E-1270F018751C}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -22262,4 +22237,29 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F5CFE981-CBAC-4360-B0CE-AB3235A33930}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F919D1BA-3E11-4877-AEE4-5A5340B7B50A}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="89c54d5b-05ac-45d5-9242-aabb385cc5ad"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="f76aa77c-8923-4724-9a6d-d588cc513697"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Atualizacao de base — Tayrone incluido em metas.xlsx (FILIAL=LIN)
Com o cadastro, as 50 linhas dele (46 un, R$ 1,95 mi) passam a contar no
total da loja de Linhares. Segue INATIVO, entao nao aparece na matriz
individual — so soma para a loja, como combinado.

Vao junto: clientes.xlsx (atualizado manualmente) e o screenshot de
diagnostico do script CNH.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/dados/metas.xlsx
+++ b/dados/metas.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pedro.sa\Documents\dashboard-oportunidades\dados\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{55F1C0CF-59CA-4E66-A1C7-1C85BAE78261}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DED88F9D-4825-4696-B598-D9528DCAD3AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -18,7 +18,7 @@
     <sheet name="ORÇAMENTO" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">CONSULTOR!$A$1:$R$249</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">CONSULTOR!$A$1:$R$254</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1534" uniqueCount="95">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1554" uniqueCount="96">
   <si>
     <t>CÓD</t>
   </si>
@@ -326,6 +326,9 @@
   </si>
   <si>
     <t>RAFAEL.CAETANO</t>
+  </si>
+  <si>
+    <t>TAYRONE.SEPULCRO</t>
   </si>
 </sst>
 </file>
@@ -737,7 +740,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:R253"/>
+  <dimension ref="A1:R258"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.140625" style="4"/>
@@ -13459,7 +13462,7 @@
         <v>47</v>
       </c>
       <c r="R232" s="4" t="s">
-        <v>21</v>
+        <v>34</v>
       </c>
     </row>
     <row r="233" spans="1:18" x14ac:dyDescent="0.25">
@@ -13515,7 +13518,7 @@
         <v>47</v>
       </c>
       <c r="R233" s="4" t="s">
-        <v>21</v>
+        <v>34</v>
       </c>
     </row>
     <row r="234" spans="1:18" x14ac:dyDescent="0.25">
@@ -13571,7 +13574,7 @@
         <v>47</v>
       </c>
       <c r="R234" s="4" t="s">
-        <v>21</v>
+        <v>34</v>
       </c>
     </row>
     <row r="235" spans="1:18" x14ac:dyDescent="0.25">
@@ -13627,7 +13630,7 @@
         <v>47</v>
       </c>
       <c r="R235" s="4" t="s">
-        <v>21</v>
+        <v>34</v>
       </c>
     </row>
     <row r="236" spans="1:18" x14ac:dyDescent="0.25">
@@ -13683,7 +13686,7 @@
         <v>47</v>
       </c>
       <c r="R236" s="4" t="s">
-        <v>21</v>
+        <v>34</v>
       </c>
     </row>
     <row r="237" spans="1:18" x14ac:dyDescent="0.25">
@@ -13739,7 +13742,7 @@
         <v>47</v>
       </c>
       <c r="R237" s="4" t="s">
-        <v>21</v>
+        <v>34</v>
       </c>
     </row>
     <row r="238" spans="1:18" x14ac:dyDescent="0.25">
@@ -13795,7 +13798,7 @@
         <v>47</v>
       </c>
       <c r="R238" s="4" t="s">
-        <v>21</v>
+        <v>34</v>
       </c>
     </row>
     <row r="239" spans="1:18" x14ac:dyDescent="0.25">
@@ -13851,68 +13854,62 @@
         <v>47</v>
       </c>
       <c r="R239" s="4" t="s">
-        <v>21</v>
+        <v>34</v>
       </c>
     </row>
     <row r="240" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A240" s="4">
-        <v>250111</v>
+        <v>220999</v>
       </c>
       <c r="B240" s="4" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="C240" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="G240" s="4">
-        <v>0</v>
+        <v>23</v>
       </c>
       <c r="H240" s="4">
         <v>0</v>
       </c>
       <c r="I240" s="4">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J240" s="4">
         <v>0</v>
       </c>
       <c r="K240" s="4">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L240" s="4">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M240" s="4">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="N240" s="4">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O240" s="4">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="P240" s="4">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="Q240" s="4" t="s">
-        <v>38</v>
+        <v>47</v>
       </c>
       <c r="R240" s="4" t="s">
-        <v>21</v>
+        <v>34</v>
       </c>
     </row>
     <row r="241" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A241" s="4">
-        <v>250111</v>
+        <v>220999</v>
       </c>
       <c r="B241" s="4" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="C241" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="G241" s="4">
-        <v>1</v>
+        <v>24</v>
       </c>
       <c r="H241" s="4">
         <v>1</v>
@@ -13924,151 +13921,144 @@
         <v>1</v>
       </c>
       <c r="K241" s="4">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L241" s="4">
         <v>1</v>
       </c>
       <c r="M241" s="4">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N241" s="4">
         <v>1</v>
       </c>
       <c r="O241" s="4">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P241" s="4">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="Q241" s="4" t="s">
-        <v>38</v>
+        <v>47</v>
       </c>
       <c r="R241" s="4" t="s">
-        <v>21</v>
+        <v>34</v>
       </c>
     </row>
     <row r="242" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A242" s="4">
-        <v>250111</v>
+        <v>220999</v>
       </c>
       <c r="B242" s="4" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="C242" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="G242" s="4">
-        <v>0</v>
+        <v>19</v>
       </c>
       <c r="H242" s="4">
-        <v>1</v>
+        <v>499177</v>
       </c>
       <c r="I242" s="4">
-        <v>0</v>
+        <v>327756</v>
       </c>
       <c r="J242" s="4">
-        <v>0</v>
+        <v>234504</v>
       </c>
       <c r="K242" s="4">
-        <v>1</v>
+        <v>308557</v>
       </c>
       <c r="L242" s="4">
-        <v>0</v>
+        <v>514262</v>
       </c>
       <c r="M242" s="4">
-        <v>0</v>
+        <v>455293</v>
       </c>
       <c r="N242" s="4">
-        <v>1</v>
+        <v>519748</v>
       </c>
       <c r="O242" s="4">
-        <v>0</v>
+        <v>532090</v>
       </c>
       <c r="P242" s="4">
-        <v>3</v>
+        <f>SUM(H242:O242)</f>
+        <v>3391387</v>
       </c>
       <c r="Q242" s="4" t="s">
-        <v>38</v>
+        <v>47</v>
       </c>
       <c r="R242" s="4" t="s">
-        <v>21</v>
+        <v>34</v>
       </c>
     </row>
     <row r="243" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A243" s="4">
-        <v>250111</v>
+        <v>220999</v>
       </c>
       <c r="B243" s="4" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="C243" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="H243" s="4">
+        <v>2</v>
+      </c>
+      <c r="I243" s="4">
+        <v>3</v>
+      </c>
+      <c r="J243" s="4">
+        <v>2</v>
+      </c>
+      <c r="K243" s="4">
+        <v>3</v>
+      </c>
+      <c r="L243" s="4">
+        <v>3</v>
+      </c>
+      <c r="M243" s="4">
+        <v>2</v>
+      </c>
+      <c r="N243" s="4">
+        <v>2</v>
+      </c>
+      <c r="O243" s="4">
+        <v>2</v>
+      </c>
+      <c r="P243" s="4">
+        <f>SUM(H243:O243)</f>
         <v>19</v>
       </c>
-      <c r="G243" s="4">
-        <v>70000</v>
-      </c>
-      <c r="H243" s="4">
-        <v>70000</v>
-      </c>
-      <c r="I243" s="4">
-        <v>90000</v>
-      </c>
-      <c r="J243" s="4">
-        <v>90000</v>
-      </c>
-      <c r="K243" s="4">
-        <v>120000</v>
-      </c>
-      <c r="L243" s="4">
-        <v>100000</v>
-      </c>
-      <c r="M243" s="4">
-        <v>120000</v>
-      </c>
-      <c r="N243" s="4">
-        <v>70000</v>
-      </c>
-      <c r="O243" s="4">
-        <v>70000</v>
-      </c>
-      <c r="P243" s="4">
-        <v>800000</v>
-      </c>
       <c r="Q243" s="4" t="s">
-        <v>38</v>
+        <v>47</v>
       </c>
       <c r="R243" s="4" t="s">
-        <v>21</v>
+        <v>34</v>
       </c>
     </row>
     <row r="244" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A244" s="4">
-        <v>250111</v>
+        <v>220999</v>
       </c>
       <c r="B244" s="4" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="C244" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="G244" s="4">
-        <v>0</v>
+        <v>39</v>
       </c>
       <c r="H244" s="4">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I244" s="4">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J244" s="4">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K244" s="4">
         <v>0</v>
       </c>
       <c r="L244" s="4">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M244" s="4">
         <v>0</v>
@@ -14080,13 +14070,13 @@
         <v>0</v>
       </c>
       <c r="P244" s="4">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="Q244" s="4" t="s">
-        <v>38</v>
+        <v>47</v>
       </c>
       <c r="R244" s="4" t="s">
-        <v>21</v>
+        <v>34</v>
       </c>
     </row>
     <row r="245" spans="1:18" x14ac:dyDescent="0.25">
@@ -14097,7 +14087,7 @@
         <v>92</v>
       </c>
       <c r="C245" s="4" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="G245" s="4">
         <v>0</v>
@@ -14144,22 +14134,22 @@
         <v>92</v>
       </c>
       <c r="C246" s="4" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="G246" s="4">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H246" s="4">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I246" s="4">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J246" s="4">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K246" s="4">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L246" s="4">
         <v>1</v>
@@ -14168,13 +14158,13 @@
         <v>1</v>
       </c>
       <c r="N246" s="4">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O246" s="4">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P246" s="4">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="Q246" s="4" t="s">
         <v>38</v>
@@ -14191,37 +14181,37 @@
         <v>92</v>
       </c>
       <c r="C247" s="4" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="G247" s="4">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H247" s="4">
         <v>1</v>
       </c>
       <c r="I247" s="4">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J247" s="4">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K247" s="4">
         <v>1</v>
       </c>
       <c r="L247" s="4">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M247" s="4">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N247" s="4">
         <v>1</v>
       </c>
       <c r="O247" s="4">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P247" s="4">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="Q247" s="4" t="s">
         <v>38</v>
@@ -14238,37 +14228,37 @@
         <v>92</v>
       </c>
       <c r="C248" s="4" t="s">
-        <v>29</v>
+        <v>19</v>
       </c>
       <c r="G248" s="4">
-        <v>0</v>
+        <v>70000</v>
       </c>
       <c r="H248" s="4">
-        <v>200000</v>
+        <v>70000</v>
       </c>
       <c r="I248" s="4">
-        <v>0</v>
+        <v>90000</v>
       </c>
       <c r="J248" s="4">
-        <v>400000</v>
+        <v>90000</v>
       </c>
       <c r="K248" s="4">
-        <v>0</v>
+        <v>120000</v>
       </c>
       <c r="L248" s="4">
-        <v>200000</v>
+        <v>100000</v>
       </c>
       <c r="M248" s="4">
-        <v>0</v>
+        <v>120000</v>
       </c>
       <c r="N248" s="4">
-        <v>500000</v>
+        <v>70000</v>
       </c>
       <c r="O248" s="4">
-        <v>200000</v>
+        <v>70000</v>
       </c>
       <c r="P248" s="4">
-        <v>1500000</v>
+        <v>800000</v>
       </c>
       <c r="Q248" s="4" t="s">
         <v>38</v>
@@ -14285,19 +14275,19 @@
         <v>92</v>
       </c>
       <c r="C249" s="4" t="s">
-        <v>39</v>
+        <v>25</v>
       </c>
       <c r="G249" s="4">
         <v>0</v>
       </c>
       <c r="H249" s="4">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I249" s="4">
         <v>0</v>
       </c>
       <c r="J249" s="4">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K249" s="4">
         <v>0</v>
@@ -14306,16 +14296,16 @@
         <v>0</v>
       </c>
       <c r="M249" s="4">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N249" s="4">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O249" s="4">
         <v>0</v>
       </c>
       <c r="P249" s="4">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="Q249" s="4" t="s">
         <v>38</v>
@@ -14326,13 +14316,25 @@
     </row>
     <row r="250" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A250" s="4">
-        <v>40011</v>
+        <v>250111</v>
       </c>
       <c r="B250" s="4" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="C250" s="4" t="s">
-        <v>23</v>
+        <v>26</v>
+      </c>
+      <c r="G250" s="4">
+        <v>0</v>
+      </c>
+      <c r="H250" s="4">
+        <v>0</v>
+      </c>
+      <c r="I250" s="4">
+        <v>2</v>
+      </c>
+      <c r="J250" s="4">
+        <v>0</v>
       </c>
       <c r="K250" s="4">
         <v>0</v>
@@ -14341,19 +14343,19 @@
         <v>0</v>
       </c>
       <c r="M250" s="4">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N250" s="4">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="O250" s="4">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P250" s="4">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="Q250" s="4" t="s">
-        <v>32</v>
+        <v>38</v>
       </c>
       <c r="R250" s="4" t="s">
         <v>21</v>
@@ -14361,19 +14363,31 @@
     </row>
     <row r="251" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A251" s="4">
-        <v>40011</v>
+        <v>250111</v>
       </c>
       <c r="B251" s="4" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="C251" s="4" t="s">
-        <v>24</v>
+        <v>27</v>
+      </c>
+      <c r="G251" s="4">
+        <v>0</v>
+      </c>
+      <c r="H251" s="4">
+        <v>0</v>
+      </c>
+      <c r="I251" s="4">
+        <v>0</v>
+      </c>
+      <c r="J251" s="4">
+        <v>0</v>
       </c>
       <c r="K251" s="4">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L251" s="4">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M251" s="4">
         <v>1</v>
@@ -14382,13 +14396,13 @@
         <v>0</v>
       </c>
       <c r="O251" s="4">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P251" s="4">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="Q251" s="4" t="s">
-        <v>32</v>
+        <v>38</v>
       </c>
       <c r="R251" s="4" t="s">
         <v>21</v>
@@ -14396,34 +14410,46 @@
     </row>
     <row r="252" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A252" s="4">
-        <v>40011</v>
+        <v>250111</v>
       </c>
       <c r="B252" s="4" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="C252" s="4" t="s">
-        <v>19</v>
+        <v>28</v>
+      </c>
+      <c r="G252" s="4">
+        <v>1</v>
+      </c>
+      <c r="H252" s="4">
+        <v>1</v>
+      </c>
+      <c r="I252" s="4">
+        <v>1</v>
+      </c>
+      <c r="J252" s="4">
+        <v>1</v>
       </c>
       <c r="K252" s="4">
-        <v>100000</v>
+        <v>1</v>
       </c>
       <c r="L252" s="4">
-        <v>150000</v>
+        <v>1</v>
       </c>
       <c r="M252" s="4">
-        <v>140000</v>
+        <v>1</v>
       </c>
       <c r="N252" s="4">
-        <v>120000</v>
+        <v>1</v>
       </c>
       <c r="O252" s="4">
-        <v>80000</v>
+        <v>1</v>
       </c>
       <c r="P252" s="4">
-        <v>590000</v>
+        <v>9</v>
       </c>
       <c r="Q252" s="4" t="s">
-        <v>32</v>
+        <v>38</v>
       </c>
       <c r="R252" s="4" t="s">
         <v>21</v>
@@ -14431,42 +14457,242 @@
     </row>
     <row r="253" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A253" s="4">
-        <v>40011</v>
+        <v>250111</v>
       </c>
       <c r="B253" s="4" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="C253" s="4" t="s">
-        <v>28</v>
+        <v>29</v>
+      </c>
+      <c r="G253" s="4">
+        <v>0</v>
+      </c>
+      <c r="H253" s="4">
+        <v>200000</v>
+      </c>
+      <c r="I253" s="4">
+        <v>0</v>
+      </c>
+      <c r="J253" s="4">
+        <v>400000</v>
       </c>
       <c r="K253" s="4">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L253" s="4">
-        <v>2</v>
+        <v>200000</v>
       </c>
       <c r="M253" s="4">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N253" s="4">
-        <v>1</v>
+        <v>500000</v>
       </c>
       <c r="O253" s="4">
-        <v>1</v>
+        <v>200000</v>
       </c>
       <c r="P253" s="4">
-        <v>6</v>
+        <v>1500000</v>
       </c>
       <c r="Q253" s="4" t="s">
-        <v>32</v>
+        <v>38</v>
       </c>
       <c r="R253" s="4" t="s">
         <v>21</v>
       </c>
     </row>
+    <row r="254" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A254" s="4">
+        <v>250111</v>
+      </c>
+      <c r="B254" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="C254" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="G254" s="4">
+        <v>0</v>
+      </c>
+      <c r="H254" s="4">
+        <v>1</v>
+      </c>
+      <c r="I254" s="4">
+        <v>0</v>
+      </c>
+      <c r="J254" s="4">
+        <v>1</v>
+      </c>
+      <c r="K254" s="4">
+        <v>0</v>
+      </c>
+      <c r="L254" s="4">
+        <v>0</v>
+      </c>
+      <c r="M254" s="4">
+        <v>1</v>
+      </c>
+      <c r="N254" s="4">
+        <v>0</v>
+      </c>
+      <c r="O254" s="4">
+        <v>0</v>
+      </c>
+      <c r="P254" s="4">
+        <v>3</v>
+      </c>
+      <c r="Q254" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="R254" s="4" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="255" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A255" s="4">
+        <v>40011</v>
+      </c>
+      <c r="B255" s="4" t="s">
+        <v>93</v>
+      </c>
+      <c r="C255" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="K255" s="4">
+        <v>0</v>
+      </c>
+      <c r="L255" s="4">
+        <v>0</v>
+      </c>
+      <c r="M255" s="4">
+        <v>1</v>
+      </c>
+      <c r="N255" s="4">
+        <v>0</v>
+      </c>
+      <c r="O255" s="4">
+        <v>1</v>
+      </c>
+      <c r="P255" s="4">
+        <v>2</v>
+      </c>
+      <c r="Q255" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="R255" s="4" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="256" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A256" s="4">
+        <v>40011</v>
+      </c>
+      <c r="B256" s="4" t="s">
+        <v>93</v>
+      </c>
+      <c r="C256" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="K256" s="4">
+        <v>1</v>
+      </c>
+      <c r="L256" s="4">
+        <v>0</v>
+      </c>
+      <c r="M256" s="4">
+        <v>1</v>
+      </c>
+      <c r="N256" s="4">
+        <v>0</v>
+      </c>
+      <c r="O256" s="4">
+        <v>1</v>
+      </c>
+      <c r="P256" s="4">
+        <v>3</v>
+      </c>
+      <c r="Q256" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="R256" s="4" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="257" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A257" s="4">
+        <v>40011</v>
+      </c>
+      <c r="B257" s="4" t="s">
+        <v>93</v>
+      </c>
+      <c r="C257" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="K257" s="4">
+        <v>100000</v>
+      </c>
+      <c r="L257" s="4">
+        <v>150000</v>
+      </c>
+      <c r="M257" s="4">
+        <v>140000</v>
+      </c>
+      <c r="N257" s="4">
+        <v>120000</v>
+      </c>
+      <c r="O257" s="4">
+        <v>80000</v>
+      </c>
+      <c r="P257" s="4">
+        <v>590000</v>
+      </c>
+      <c r="Q257" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="R257" s="4" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="258" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A258" s="4">
+        <v>40011</v>
+      </c>
+      <c r="B258" s="4" t="s">
+        <v>93</v>
+      </c>
+      <c r="C258" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="K258" s="4">
+        <v>1</v>
+      </c>
+      <c r="L258" s="4">
+        <v>2</v>
+      </c>
+      <c r="M258" s="4">
+        <v>1</v>
+      </c>
+      <c r="N258" s="4">
+        <v>1</v>
+      </c>
+      <c r="O258" s="4">
+        <v>1</v>
+      </c>
+      <c r="P258" s="4">
+        <v>6</v>
+      </c>
+      <c r="Q258" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="R258" s="4" t="s">
+        <v>21</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:R249" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:R254" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -22006,6 +22232,26 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="f76aa77c-8923-4724-9a6d-d588cc513697">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="89c54d5b-05ac-45d5-9242-aabb385cc5ad" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100B96036E30F13644F923D207E371C305D" ma:contentTypeVersion="11" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="1d197ceb99055fd1a93a3a14aec1bdd8">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="f76aa77c-8923-4724-9a6d-d588cc513697" xmlns:ns3="89c54d5b-05ac-45d5-9242-aabb385cc5ad" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="5b86266bfd619f312673123d0bd20d23" ns2:_="" ns3:_="">
     <xsd:import namespace="f76aa77c-8923-4724-9a6d-d588cc513697"/>
@@ -22200,27 +22446,32 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F919D1BA-3E11-4877-AEE4-5A5340B7B50A}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="89c54d5b-05ac-45d5-9242-aabb385cc5ad"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="f76aa77c-8923-4724-9a6d-d588cc513697"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="f76aa77c-8923-4724-9a6d-d588cc513697">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="89c54d5b-05ac-45d5-9242-aabb385cc5ad" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F5CFE981-CBAC-4360-B0CE-AB3235A33930}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8BDC8EFC-C946-4B3C-B84E-1270F018751C}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -22237,29 +22488,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F5CFE981-CBAC-4360-B0CE-AB3235A33930}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F919D1BA-3E11-4877-AEE4-5A5340B7B50A}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="89c54d5b-05ac-45d5-9242-aabb385cc5ad"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="f76aa77c-8923-4724-9a6d-d588cc513697"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>